<commit_message>
Updated IND_grids_kan60 model - 2026-09-29 16:36
</commit_message>
<xml_diff>
--- a/VerveStacks_IND_grids_kan60/Sets-vervestacks.xlsx
+++ b/VerveStacks_IND_grids_kan60/Sets-vervestacks.xlsx
@@ -2,26 +2,23 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="25928"/>
-  <workbookPr updateLinks="never" defaultThemeVersion="166925"/>
+  <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Veda\Veda\Veda_models\vervestacks_models\VerveStacks_IND_grids_kan60\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0CB4AE30-3474-46A6-BBFB-800B3880BFA7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{491D462D-062B-408B-8AAF-30145B3981B0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="3675" yWindow="3675" windowWidth="21600" windowHeight="11423" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="3675" yWindow="3675" windowWidth="21600" windowHeight="12773" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="VEDA_Sets-Comm" sheetId="2" r:id="rId1"/>
-    <sheet name="geo_sets" sheetId="5" r:id="rId2"/>
-    <sheet name="VEDA_Sets-Proc" sheetId="4" r:id="rId3"/>
+    <sheet name="VEDA_Sets-Comm" sheetId="1" r:id="rId1"/>
+    <sheet name="geo_sets" sheetId="2" r:id="rId2"/>
+    <sheet name="VEDA_Sets-Proc" sheetId="3" r:id="rId3"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
-      <x15:workbookPr chartTrackingRefBase="1"/>
-    </ext>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
       <xcalcf:calcFeatures>
         <xcalcf:feature name="microsoft.com:RD"/>
@@ -40,6 +37,129 @@
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1079" uniqueCount="595">
   <si>
+    <t>~TFM_Csets</t>
+  </si>
+  <si>
+    <t>CSET_SET</t>
+  </si>
+  <si>
+    <t>CSET_CN</t>
+  </si>
+  <si>
+    <t>CSET_CD</t>
+  </si>
+  <si>
+    <t>SetName</t>
+  </si>
+  <si>
+    <t>SetDesc</t>
+  </si>
+  <si>
+    <t>c_Pos_AndOr</t>
+  </si>
+  <si>
+    <t>c_Neg_AndOr</t>
+  </si>
+  <si>
+    <t>Comment</t>
+  </si>
+  <si>
+    <t>e*spv*</t>
+  </si>
+  <si>
+    <t>Solar elec</t>
+  </si>
+  <si>
+    <t>e*won*,e*wof*</t>
+  </si>
+  <si>
+    <t>Wind elec</t>
+  </si>
+  <si>
+    <t>coal,gas,oil</t>
+  </si>
+  <si>
+    <t>fossil</t>
+  </si>
+  <si>
+    <t>geothermal,hydro,solar,wind</t>
+  </si>
+  <si>
+    <t>renewable</t>
+  </si>
+  <si>
+    <t>bioenergy</t>
+  </si>
+  <si>
+    <t>hydrogen</t>
+  </si>
+  <si>
+    <t>nuclear</t>
+  </si>
+  <si>
+    <t>ELC,e[_]*</t>
+  </si>
+  <si>
+    <t>Electricity</t>
+  </si>
+  <si>
+    <t>elc_buildings</t>
+  </si>
+  <si>
+    <t>buildings</t>
+  </si>
+  <si>
+    <t>elc_industry</t>
+  </si>
+  <si>
+    <t>industry</t>
+  </si>
+  <si>
+    <t>elc_transport</t>
+  </si>
+  <si>
+    <t>transport</t>
+  </si>
+  <si>
+    <t>elc_roadtransport</t>
+  </si>
+  <si>
+    <t>EVs</t>
+  </si>
+  <si>
+    <t>co2</t>
+  </si>
+  <si>
+    <t>co2captured,co2[_]*</t>
+  </si>
+  <si>
+    <t>CO2Captured</t>
+  </si>
+  <si>
+    <t>co2s[_]*</t>
+  </si>
+  <si>
+    <t>CO2Stored</t>
+  </si>
+  <si>
+    <t>~tfm_psets</t>
+  </si>
+  <si>
+    <t>setname</t>
+  </si>
+  <si>
+    <t>pset_co</t>
+  </si>
+  <si>
+    <t>pset_ci</t>
+  </si>
+  <si>
+    <t>t_pos_andor</t>
+  </si>
+  <si>
+    <t>OR</t>
+  </si>
+  <si>
     <t>~TFM_Psets</t>
   </si>
   <si>
@@ -58,463 +178,340 @@
     <t>PSET_CO</t>
   </si>
   <si>
-    <t>SetName</t>
-  </si>
-  <si>
-    <t>SetDesc</t>
-  </si>
-  <si>
     <t>T_Pos_AndOr</t>
   </si>
   <si>
     <t>T_Neg_AndOr</t>
   </si>
   <si>
-    <t>Comment</t>
-  </si>
-  <si>
     <t>ELE</t>
   </si>
   <si>
-    <t>~TFM_Csets</t>
-  </si>
-  <si>
-    <t>CSET_SET</t>
-  </si>
-  <si>
-    <t>CSET_CN</t>
-  </si>
-  <si>
-    <t>CSET_CD</t>
-  </si>
-  <si>
-    <t>c_Pos_AndOr</t>
-  </si>
-  <si>
-    <t>c_Neg_AndOr</t>
+    <t>EP_GAS-CC*,EP_OIL-CC*,*gas_cc*,*gas_comb*,*ember</t>
+  </si>
+  <si>
+    <t>gas,elcnga,elcgas,oil,elco</t>
   </si>
   <si>
     <t>CCGT</t>
   </si>
   <si>
+    <t>Combined Cycle Gas Turbine</t>
+  </si>
+  <si>
+    <t>Ramp ~8%/min</t>
+  </si>
+  <si>
+    <t>EP_GAS-GT*,EP_OIL-GT*,*gas_turbine*,EN*CT*</t>
+  </si>
+  <si>
+    <t>OCGT</t>
+  </si>
+  <si>
+    <t>Open Cycle Gas Turbine (Peaker)</t>
+  </si>
+  <si>
+    <t>Ramp ~15%/min</t>
+  </si>
+  <si>
+    <t>EP_GAS-ST*,EP_OIL-ST*,*steam*</t>
+  </si>
+  <si>
+    <t>Gas_Oil_Steam</t>
+  </si>
+  <si>
+    <t>Gas/Oil Steam Turbine</t>
+  </si>
+  <si>
+    <t>EP_GAS-IC*,EP_OIL-IC*,*gas_engine*,*internal_comb*</t>
+  </si>
+  <si>
+    <t>Int_Comb</t>
+  </si>
+  <si>
+    <t>Internal Combustion Engine</t>
+  </si>
+  <si>
+    <t>EP_COA-ST*,EP_LIG-ST*,*-CFB*,*coal_st*,*coal_subcritical*</t>
+  </si>
+  <si>
+    <t>coal,elcco*</t>
+  </si>
+  <si>
+    <t>Subcrit_Coal</t>
+  </si>
+  <si>
     <t>Subcritical Coal</t>
   </si>
   <si>
+    <t>Ramp ~3%/min</t>
+  </si>
+  <si>
+    <t>EP_COA-SC*,EP_COA-USC*,EP_LIG-SC*,EP_LIG-USC*,*coal_sc*,*coal_usc*,*coal_supercritical*,*coal_ultrasupercritical*</t>
+  </si>
+  <si>
+    <t>Supercrit_Coal</t>
+  </si>
+  <si>
+    <t>Supercritical/Ultra-Supercritical Coal</t>
+  </si>
+  <si>
+    <t>Ramp ~4%/min</t>
+  </si>
+  <si>
+    <t>*-IGCC*,*coal_igcc*</t>
+  </si>
+  <si>
+    <t>IGCC</t>
+  </si>
+  <si>
+    <t>Integrated Gasification CC</t>
+  </si>
+  <si>
+    <t>CHP</t>
+  </si>
+  <si>
+    <t>CHP_Gas</t>
+  </si>
+  <si>
+    <t>Gas/Oil CHP</t>
+  </si>
+  <si>
+    <t>Same ramp as ELE counterpart</t>
+  </si>
+  <si>
+    <t>CHP_Coal</t>
+  </si>
+  <si>
+    <t>Coal CHP</t>
+  </si>
+  <si>
+    <t>bio*,elcb*</t>
+  </si>
+  <si>
+    <t>CHP_Bio</t>
+  </si>
+  <si>
+    <t>Biomass CHP</t>
+  </si>
+  <si>
+    <t>HPL</t>
+  </si>
+  <si>
+    <t>HOP_Gas</t>
+  </si>
+  <si>
+    <t>Gas/Oil Heat-Only Boiler</t>
+  </si>
+  <si>
+    <t>HOP_Bio</t>
+  </si>
+  <si>
+    <t>Biomass Heat-Only Boiler</t>
+  </si>
+  <si>
+    <t>-*HP*</t>
+  </si>
+  <si>
+    <t>elc,e[_]*</t>
+  </si>
+  <si>
+    <t>HOP_Elec</t>
+  </si>
+  <si>
+    <t>Electric Boiler (DH)</t>
+  </si>
+  <si>
+    <t>*HP*</t>
+  </si>
+  <si>
+    <t>Heat_Pump</t>
+  </si>
+  <si>
+    <t>Large-Scale Heat Pump</t>
+  </si>
+  <si>
+    <t>Bio_Power</t>
+  </si>
+  <si>
+    <t>Biomass Power (ELE)</t>
+  </si>
+  <si>
+    <t>ELE,CHP</t>
+  </si>
+  <si>
+    <t>elcs*,solar</t>
+  </si>
+  <si>
+    <t>Solar_Util</t>
+  </si>
+  <si>
+    <t>Solar Utility</t>
+  </si>
+  <si>
+    <t>elcwin,windon</t>
+  </si>
+  <si>
+    <t>Wind_Onshore</t>
+  </si>
+  <si>
+    <t>Wind Onshore</t>
+  </si>
+  <si>
+    <t>windoff</t>
+  </si>
+  <si>
+    <t>Wind_Offshore</t>
+  </si>
+  <si>
+    <t>Wind Offshore</t>
+  </si>
+  <si>
+    <t>elcgeo,geothermal</t>
+  </si>
+  <si>
+    <t>Geothermal</t>
+  </si>
+  <si>
+    <t>Geothermal Power</t>
+  </si>
+  <si>
+    <t>-*ror*</t>
+  </si>
+  <si>
+    <t>elchyd,hydro</t>
+  </si>
+  <si>
+    <t>Hydro_Dam</t>
+  </si>
+  <si>
+    <t>Hydro Dam</t>
+  </si>
+  <si>
+    <t>And</t>
+  </si>
+  <si>
+    <t>Or</t>
+  </si>
+  <si>
+    <t>*HYD-ROR*,*ror*</t>
+  </si>
+  <si>
+    <t>Hydro_RoR</t>
+  </si>
+  <si>
+    <t>Hydro Run-of-River</t>
+  </si>
+  <si>
+    <t>-*SMR*</t>
+  </si>
+  <si>
+    <t>elcnuc,nuclear</t>
+  </si>
+  <si>
+    <t>Nuclear_P</t>
+  </si>
+  <si>
+    <t>Nuclear (Conventional)</t>
+  </si>
+  <si>
+    <t>*SMR*</t>
+  </si>
+  <si>
+    <t>Nuclear_SMR</t>
+  </si>
+  <si>
+    <t>Nuclear SMR</t>
+  </si>
+  <si>
     <t>STG</t>
   </si>
   <si>
-    <t>IGCC</t>
+    <t>*HPS*,*hydro_ps*</t>
+  </si>
+  <si>
+    <t>Hydro_PS</t>
+  </si>
+  <si>
+    <t>Pumped Hydro Storage</t>
+  </si>
+  <si>
+    <t>*4h*,*8h*,*12h*,-*EV*</t>
+  </si>
+  <si>
+    <t>Batt_Util</t>
+  </si>
+  <si>
+    <t>Utility Battery Storage</t>
   </si>
   <si>
     <t>*EV*</t>
   </si>
   <si>
+    <t>Batt_EV</t>
+  </si>
+  <si>
+    <t>EV Battery</t>
+  </si>
+  <si>
+    <t>IRE</t>
+  </si>
+  <si>
+    <t>g[_]*</t>
+  </si>
+  <si>
+    <t>Grid</t>
+  </si>
+  <si>
+    <t>DMD</t>
+  </si>
+  <si>
+    <t>Demand</t>
+  </si>
+  <si>
+    <t>PRE</t>
+  </si>
+  <si>
+    <t>stepdown*</t>
+  </si>
+  <si>
+    <t>Transformers Dn</t>
+  </si>
+  <si>
+    <t>stepup*</t>
+  </si>
+  <si>
+    <t>Transformers Up</t>
+  </si>
+  <si>
+    <t>distr*</t>
+  </si>
+  <si>
+    <t>Aggregators</t>
+  </si>
+  <si>
+    <t>IMP*Z</t>
+  </si>
+  <si>
+    <t>DUMMY_IMP</t>
+  </si>
+  <si>
+    <t>distr_sol*</t>
+  </si>
+  <si>
+    <t>distr_won*</t>
+  </si>
+  <si>
+    <t>distr_wof*</t>
+  </si>
+  <si>
     <t>geothermal</t>
   </si>
   <si>
     <t>hydro</t>
   </si>
   <si>
-    <t>nuclear</t>
-  </si>
-  <si>
-    <t>And</t>
-  </si>
-  <si>
-    <t>Or</t>
-  </si>
-  <si>
-    <t>Grid</t>
-  </si>
-  <si>
-    <t>IRE</t>
-  </si>
-  <si>
-    <t>g[_]*</t>
-  </si>
-  <si>
-    <t>DMD</t>
-  </si>
-  <si>
-    <t>Demand</t>
-  </si>
-  <si>
-    <t>e*spv*</t>
-  </si>
-  <si>
-    <t>e*won*,e*wof*</t>
-  </si>
-  <si>
-    <t>bioenergy</t>
-  </si>
-  <si>
-    <t>hydrogen</t>
-  </si>
-  <si>
-    <t>elc_buildings</t>
-  </si>
-  <si>
-    <t>elc_industry</t>
-  </si>
-  <si>
-    <t>elc_transport</t>
-  </si>
-  <si>
-    <t>elc_roadtransport</t>
-  </si>
-  <si>
-    <t>co2</t>
-  </si>
-  <si>
-    <t>buildings</t>
-  </si>
-  <si>
-    <t>industry</t>
-  </si>
-  <si>
-    <t>transport</t>
-  </si>
-  <si>
-    <t>EVs</t>
-  </si>
-  <si>
-    <t>fossil</t>
-  </si>
-  <si>
-    <t>coal,gas,oil</t>
-  </si>
-  <si>
-    <t>geothermal,hydro,solar,wind</t>
-  </si>
-  <si>
-    <t>PRE</t>
-  </si>
-  <si>
-    <t>stepdown*</t>
-  </si>
-  <si>
-    <t>Nuclear SMR</t>
-  </si>
-  <si>
-    <t>*SMR*</t>
-  </si>
-  <si>
-    <t>-*SMR*</t>
-  </si>
-  <si>
-    <t>Hydro Dam</t>
-  </si>
-  <si>
-    <t>renewable</t>
-  </si>
-  <si>
-    <t>Solar elec</t>
-  </si>
-  <si>
-    <t>Wind elec</t>
-  </si>
-  <si>
-    <t>Aggregators</t>
-  </si>
-  <si>
-    <t>IMP*Z</t>
-  </si>
-  <si>
-    <t>DUMMY_IMP</t>
-  </si>
-  <si>
-    <t>stepup*</t>
-  </si>
-  <si>
-    <t>Transformers Up</t>
-  </si>
-  <si>
-    <t>Transformers Dn</t>
-  </si>
-  <si>
-    <t>windoff</t>
-  </si>
-  <si>
-    <t>distr*</t>
-  </si>
-  <si>
-    <t>ELE,CHP</t>
-  </si>
-  <si>
-    <t>distr_sol*</t>
-  </si>
-  <si>
-    <t>distr_won*</t>
-  </si>
-  <si>
-    <t>distr_wof*</t>
-  </si>
-  <si>
     <t>coal</t>
-  </si>
-  <si>
-    <t>*4h*,*8h*,*12h*,-*EV*</t>
-  </si>
-  <si>
-    <t>Combined Cycle Gas Turbine</t>
-  </si>
-  <si>
-    <t>Ramp ~8%/min</t>
-  </si>
-  <si>
-    <t>OCGT</t>
-  </si>
-  <si>
-    <t>Open Cycle Gas Turbine (Peaker)</t>
-  </si>
-  <si>
-    <t>Ramp ~15%/min</t>
-  </si>
-  <si>
-    <t>Gas_Oil_Steam</t>
-  </si>
-  <si>
-    <t>Gas/Oil Steam Turbine</t>
-  </si>
-  <si>
-    <t>Int_Comb</t>
-  </si>
-  <si>
-    <t>Internal Combustion Engine</t>
-  </si>
-  <si>
-    <t>Subcrit_Coal</t>
-  </si>
-  <si>
-    <t>Ramp ~3%/min</t>
-  </si>
-  <si>
-    <t>Supercrit_Coal</t>
-  </si>
-  <si>
-    <t>Supercritical/Ultra-Supercritical Coal</t>
-  </si>
-  <si>
-    <t>Ramp ~4%/min</t>
-  </si>
-  <si>
-    <t>*-IGCC*,*coal_igcc*</t>
-  </si>
-  <si>
-    <t>Integrated Gasification CC</t>
-  </si>
-  <si>
-    <t>CHP</t>
-  </si>
-  <si>
-    <t>CHP_Gas</t>
-  </si>
-  <si>
-    <t>Gas/Oil CHP</t>
-  </si>
-  <si>
-    <t>Same ramp as ELE counterpart</t>
-  </si>
-  <si>
-    <t>CHP_Coal</t>
-  </si>
-  <si>
-    <t>Coal CHP</t>
-  </si>
-  <si>
-    <t>CHP_Bio</t>
-  </si>
-  <si>
-    <t>Biomass CHP</t>
-  </si>
-  <si>
-    <t>HPL</t>
-  </si>
-  <si>
-    <t>HOP_Gas</t>
-  </si>
-  <si>
-    <t>Gas/Oil Heat-Only Boiler</t>
-  </si>
-  <si>
-    <t>HOP_Bio</t>
-  </si>
-  <si>
-    <t>Biomass Heat-Only Boiler</t>
-  </si>
-  <si>
-    <t>HOP_Elec</t>
-  </si>
-  <si>
-    <t>Electric Boiler (DH)</t>
-  </si>
-  <si>
-    <t>Heat_Pump</t>
-  </si>
-  <si>
-    <t>Large-Scale Heat Pump</t>
-  </si>
-  <si>
-    <t>Bio_Power</t>
-  </si>
-  <si>
-    <t>Biomass Power (ELE)</t>
-  </si>
-  <si>
-    <t>elcs*,solar</t>
-  </si>
-  <si>
-    <t>Solar_Util</t>
-  </si>
-  <si>
-    <t>Solar Utility</t>
-  </si>
-  <si>
-    <t>elcwin,windon</t>
-  </si>
-  <si>
-    <t>Wind_Onshore</t>
-  </si>
-  <si>
-    <t>Wind Onshore</t>
-  </si>
-  <si>
-    <t>Wind_Offshore</t>
-  </si>
-  <si>
-    <t>Wind Offshore</t>
-  </si>
-  <si>
-    <t>elcgeo,geothermal</t>
-  </si>
-  <si>
-    <t>Geothermal</t>
-  </si>
-  <si>
-    <t>Geothermal Power</t>
-  </si>
-  <si>
-    <t>elchyd,hydro</t>
-  </si>
-  <si>
-    <t>Hydro_Dam</t>
-  </si>
-  <si>
-    <t>*HYD-ROR*,*ror*</t>
-  </si>
-  <si>
-    <t>Hydro_RoR</t>
-  </si>
-  <si>
-    <t>Hydro Run-of-River</t>
-  </si>
-  <si>
-    <t>elcnuc,nuclear</t>
-  </si>
-  <si>
-    <t>Nuclear (Conventional)</t>
-  </si>
-  <si>
-    <t>Nuclear_SMR</t>
-  </si>
-  <si>
-    <t>*HPS*,*hydro_ps*</t>
-  </si>
-  <si>
-    <t>Hydro_PS</t>
-  </si>
-  <si>
-    <t>Pumped Hydro Storage</t>
-  </si>
-  <si>
-    <t>Batt_Util</t>
-  </si>
-  <si>
-    <t>Utility Battery Storage</t>
-  </si>
-  <si>
-    <t>Batt_EV</t>
-  </si>
-  <si>
-    <t>EV Battery</t>
-  </si>
-  <si>
-    <t>EP_GAS-GT*,EP_OIL-GT*,*gas_turbine*,EN*CT*</t>
-  </si>
-  <si>
-    <t>EP_COA-ST*,EP_LIG-ST*,*-CFB*,*coal_subcritical*</t>
-  </si>
-  <si>
-    <t>co2captured,co2[_]*</t>
-  </si>
-  <si>
-    <t>CO2Captured</t>
-  </si>
-  <si>
-    <t>co2s[_]*</t>
-  </si>
-  <si>
-    <t>CO2Stored</t>
-  </si>
-  <si>
-    <t>ELC,e[_]*</t>
-  </si>
-  <si>
-    <t>Electricity</t>
-  </si>
-  <si>
-    <t>Nuclear_P</t>
-  </si>
-  <si>
-    <t>~tfm_psets</t>
-  </si>
-  <si>
-    <t>setname</t>
-  </si>
-  <si>
-    <t>pset_co</t>
-  </si>
-  <si>
-    <t>pset_ci</t>
-  </si>
-  <si>
-    <t>t_pos_andor</t>
-  </si>
-  <si>
-    <t>OR</t>
-  </si>
-  <si>
-    <t>-*ror*</t>
-  </si>
-  <si>
-    <t>EP_COA-SC*,EP_COA-USC*,EP_LIG-SC*,EP_LIG-USC*,*critical*</t>
-  </si>
-  <si>
-    <t>coal,elcco*</t>
-  </si>
-  <si>
-    <t>gas,elcnga,elcgas,oil,elco</t>
-  </si>
-  <si>
-    <t>bio*,elcb*</t>
-  </si>
-  <si>
-    <t>*HP*</t>
-  </si>
-  <si>
-    <t>-*HP*</t>
-  </si>
-  <si>
-    <t>elc,e[_]*</t>
-  </si>
-  <si>
-    <t>EP_GAS-IC*,EP_OIL-IC*,*gas_engine*,*internal_comb*</t>
-  </si>
-  <si>
-    <t>EP_GAS-CC*,EP_OIL-CC*,*gas_cc*,*gas_comb*,*ember</t>
-  </si>
-  <si>
-    <t>EP_GAS-ST*,EP_OIL-ST*,*steam*</t>
   </si>
   <si>
     <t>p_Meerut_IND</t>
@@ -1897,8 +1894,8 @@
   </borders>
   <cellStyleXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2"/>
   </cellStyleXfs>
   <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
@@ -1926,9 +1923,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - 2022 Theme">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2013 - 2022">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -1966,7 +1963,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2013 - 2022">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -2072,7 +2069,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2013 - 2022">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -2214,14 +2211,14 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme 2013 - 2022" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AB068F12-506D-4B74-BF24-03EBDA23C84D}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:H17"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
@@ -2238,70 +2235,70 @@
   <sheetData>
     <row r="1" spans="1:8" x14ac:dyDescent="0.45">
       <c r="A1" t="s">
-        <v>12</v>
+        <v>0</v>
       </c>
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.45">
       <c r="A2" t="s">
-        <v>13</v>
+        <v>1</v>
       </c>
       <c r="B2" t="s">
-        <v>14</v>
+        <v>2</v>
       </c>
       <c r="C2" t="s">
-        <v>15</v>
+        <v>3</v>
       </c>
       <c r="D2" t="s">
+        <v>4</v>
+      </c>
+      <c r="E2" t="s">
+        <v>5</v>
+      </c>
+      <c r="F2" t="s">
         <v>6</v>
       </c>
-      <c r="E2" t="s">
+      <c r="G2" t="s">
         <v>7</v>
       </c>
-      <c r="F2" t="s">
-        <v>16</v>
-      </c>
-      <c r="G2" t="s">
-        <v>17</v>
-      </c>
       <c r="H2" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.45">
       <c r="B3" t="s">
-        <v>33</v>
+        <v>9</v>
       </c>
       <c r="D3" t="s">
-        <v>56</v>
+        <v>10</v>
       </c>
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.45">
       <c r="B4" t="s">
-        <v>34</v>
+        <v>11</v>
       </c>
       <c r="D4" t="s">
-        <v>57</v>
+        <v>12</v>
       </c>
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.45">
       <c r="B5" t="s">
-        <v>47</v>
+        <v>13</v>
       </c>
       <c r="D5" t="s">
-        <v>46</v>
+        <v>14</v>
       </c>
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.45">
       <c r="B6" t="s">
-        <v>48</v>
+        <v>15</v>
       </c>
       <c r="D6" t="s">
-        <v>55</v>
+        <v>16</v>
       </c>
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.45">
       <c r="B7" t="s">
-        <v>35</v>
+        <v>17</v>
       </c>
       <c r="D7" t="str">
         <f>B7</f>
@@ -2310,7 +2307,7 @@
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.45">
       <c r="B8" t="s">
-        <v>36</v>
+        <v>18</v>
       </c>
       <c r="D8" t="str">
         <f>B8</f>
@@ -2319,7 +2316,7 @@
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.45">
       <c r="B9" t="s">
-        <v>25</v>
+        <v>19</v>
       </c>
       <c r="D9" t="str">
         <f>B9</f>
@@ -2328,47 +2325,47 @@
     </row>
     <row r="10" spans="1:8" x14ac:dyDescent="0.45">
       <c r="B10" t="s">
-        <v>139</v>
+        <v>20</v>
       </c>
       <c r="D10" t="s">
-        <v>140</v>
+        <v>21</v>
       </c>
     </row>
     <row r="11" spans="1:8" x14ac:dyDescent="0.45">
       <c r="B11" t="s">
-        <v>37</v>
+        <v>22</v>
       </c>
       <c r="D11" t="s">
-        <v>42</v>
+        <v>23</v>
       </c>
     </row>
     <row r="12" spans="1:8" x14ac:dyDescent="0.45">
       <c r="B12" t="s">
-        <v>38</v>
+        <v>24</v>
       </c>
       <c r="D12" t="s">
-        <v>43</v>
+        <v>25</v>
       </c>
     </row>
     <row r="13" spans="1:8" x14ac:dyDescent="0.45">
       <c r="B13" t="s">
-        <v>39</v>
+        <v>26</v>
       </c>
       <c r="D13" t="s">
-        <v>44</v>
+        <v>27</v>
       </c>
     </row>
     <row r="14" spans="1:8" x14ac:dyDescent="0.45">
       <c r="B14" t="s">
-        <v>40</v>
+        <v>28</v>
       </c>
       <c r="D14" t="s">
-        <v>45</v>
+        <v>29</v>
       </c>
     </row>
     <row r="15" spans="1:8" x14ac:dyDescent="0.45">
       <c r="B15" t="s">
-        <v>41</v>
+        <v>30</v>
       </c>
       <c r="D15" t="str">
         <f>B15</f>
@@ -2377,50 +2374,47 @@
     </row>
     <row r="16" spans="1:8" x14ac:dyDescent="0.45">
       <c r="B16" t="s">
-        <v>135</v>
+        <v>31</v>
       </c>
       <c r="D16" t="s">
-        <v>136</v>
+        <v>32</v>
       </c>
     </row>
     <row r="17" spans="2:4" x14ac:dyDescent="0.45">
       <c r="B17" t="s">
-        <v>137</v>
+        <v>33</v>
       </c>
       <c r="D17" t="s">
-        <v>138</v>
+        <v>34</v>
       </c>
     </row>
   </sheetData>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A5:D16">
-    <sortCondition ref="A5:A16"/>
-  </sortState>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8B9596CD-0528-4380-8F2D-D99C9A838BA1}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="B9:E228"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <sheetData>
     <row r="9" spans="2:5" x14ac:dyDescent="0.45">
       <c r="B9" t="s">
-        <v>142</v>
+        <v>35</v>
       </c>
     </row>
     <row r="10" spans="2:5" x14ac:dyDescent="0.45">
       <c r="B10" t="s">
-        <v>143</v>
+        <v>36</v>
       </c>
       <c r="C10" t="s">
-        <v>144</v>
+        <v>37</v>
       </c>
       <c r="D10" t="s">
-        <v>145</v>
+        <v>38</v>
       </c>
       <c r="E10" t="s">
-        <v>146</v>
+        <v>39</v>
       </c>
     </row>
     <row r="11" spans="2:5" x14ac:dyDescent="0.45">
@@ -2434,7 +2428,7 @@
         <v>160</v>
       </c>
       <c r="E11" t="s">
-        <v>147</v>
+        <v>40</v>
       </c>
     </row>
     <row r="12" spans="2:5" x14ac:dyDescent="0.45">
@@ -2448,7 +2442,7 @@
         <v>162</v>
       </c>
       <c r="E12" t="s">
-        <v>147</v>
+        <v>40</v>
       </c>
     </row>
     <row r="13" spans="2:5" x14ac:dyDescent="0.45">
@@ -2462,7 +2456,7 @@
         <v>164</v>
       </c>
       <c r="E13" t="s">
-        <v>147</v>
+        <v>40</v>
       </c>
     </row>
     <row r="14" spans="2:5" x14ac:dyDescent="0.45">
@@ -2476,7 +2470,7 @@
         <v>166</v>
       </c>
       <c r="E14" t="s">
-        <v>147</v>
+        <v>40</v>
       </c>
     </row>
     <row r="15" spans="2:5" x14ac:dyDescent="0.45">
@@ -2490,7 +2484,7 @@
         <v>168</v>
       </c>
       <c r="E15" t="s">
-        <v>147</v>
+        <v>40</v>
       </c>
     </row>
     <row r="16" spans="2:5" x14ac:dyDescent="0.45">
@@ -2504,7 +2498,7 @@
         <v>170</v>
       </c>
       <c r="E16" t="s">
-        <v>147</v>
+        <v>40</v>
       </c>
     </row>
     <row r="17" spans="2:5" x14ac:dyDescent="0.45">
@@ -2518,7 +2512,7 @@
         <v>172</v>
       </c>
       <c r="E17" t="s">
-        <v>147</v>
+        <v>40</v>
       </c>
     </row>
     <row r="18" spans="2:5" x14ac:dyDescent="0.45">
@@ -2532,7 +2526,7 @@
         <v>174</v>
       </c>
       <c r="E18" t="s">
-        <v>147</v>
+        <v>40</v>
       </c>
     </row>
     <row r="19" spans="2:5" x14ac:dyDescent="0.45">
@@ -2546,7 +2540,7 @@
         <v>176</v>
       </c>
       <c r="E19" t="s">
-        <v>147</v>
+        <v>40</v>
       </c>
     </row>
     <row r="20" spans="2:5" x14ac:dyDescent="0.45">
@@ -2560,7 +2554,7 @@
         <v>178</v>
       </c>
       <c r="E20" t="s">
-        <v>147</v>
+        <v>40</v>
       </c>
     </row>
     <row r="21" spans="2:5" x14ac:dyDescent="0.45">
@@ -2574,7 +2568,7 @@
         <v>180</v>
       </c>
       <c r="E21" t="s">
-        <v>147</v>
+        <v>40</v>
       </c>
     </row>
     <row r="22" spans="2:5" x14ac:dyDescent="0.45">
@@ -2588,7 +2582,7 @@
         <v>182</v>
       </c>
       <c r="E22" t="s">
-        <v>147</v>
+        <v>40</v>
       </c>
     </row>
     <row r="23" spans="2:5" x14ac:dyDescent="0.45">
@@ -2602,7 +2596,7 @@
         <v>184</v>
       </c>
       <c r="E23" t="s">
-        <v>147</v>
+        <v>40</v>
       </c>
     </row>
     <row r="24" spans="2:5" x14ac:dyDescent="0.45">
@@ -2616,7 +2610,7 @@
         <v>186</v>
       </c>
       <c r="E24" t="s">
-        <v>147</v>
+        <v>40</v>
       </c>
     </row>
     <row r="25" spans="2:5" x14ac:dyDescent="0.45">
@@ -2630,7 +2624,7 @@
         <v>188</v>
       </c>
       <c r="E25" t="s">
-        <v>147</v>
+        <v>40</v>
       </c>
     </row>
     <row r="26" spans="2:5" x14ac:dyDescent="0.45">
@@ -2644,7 +2638,7 @@
         <v>190</v>
       </c>
       <c r="E26" t="s">
-        <v>147</v>
+        <v>40</v>
       </c>
     </row>
     <row r="27" spans="2:5" x14ac:dyDescent="0.45">
@@ -2658,7 +2652,7 @@
         <v>192</v>
       </c>
       <c r="E27" t="s">
-        <v>147</v>
+        <v>40</v>
       </c>
     </row>
     <row r="28" spans="2:5" x14ac:dyDescent="0.45">
@@ -2672,7 +2666,7 @@
         <v>194</v>
       </c>
       <c r="E28" t="s">
-        <v>147</v>
+        <v>40</v>
       </c>
     </row>
     <row r="29" spans="2:5" x14ac:dyDescent="0.45">
@@ -2686,7 +2680,7 @@
         <v>196</v>
       </c>
       <c r="E29" t="s">
-        <v>147</v>
+        <v>40</v>
       </c>
     </row>
     <row r="30" spans="2:5" x14ac:dyDescent="0.45">
@@ -2700,7 +2694,7 @@
         <v>198</v>
       </c>
       <c r="E30" t="s">
-        <v>147</v>
+        <v>40</v>
       </c>
     </row>
     <row r="31" spans="2:5" x14ac:dyDescent="0.45">
@@ -2714,7 +2708,7 @@
         <v>200</v>
       </c>
       <c r="E31" t="s">
-        <v>147</v>
+        <v>40</v>
       </c>
     </row>
     <row r="32" spans="2:5" x14ac:dyDescent="0.45">
@@ -2728,7 +2722,7 @@
         <v>202</v>
       </c>
       <c r="E32" t="s">
-        <v>147</v>
+        <v>40</v>
       </c>
     </row>
     <row r="33" spans="2:5" x14ac:dyDescent="0.45">
@@ -2742,7 +2736,7 @@
         <v>204</v>
       </c>
       <c r="E33" t="s">
-        <v>147</v>
+        <v>40</v>
       </c>
     </row>
     <row r="34" spans="2:5" x14ac:dyDescent="0.45">
@@ -2756,7 +2750,7 @@
         <v>206</v>
       </c>
       <c r="E34" t="s">
-        <v>147</v>
+        <v>40</v>
       </c>
     </row>
     <row r="35" spans="2:5" x14ac:dyDescent="0.45">
@@ -2770,7 +2764,7 @@
         <v>208</v>
       </c>
       <c r="E35" t="s">
-        <v>147</v>
+        <v>40</v>
       </c>
     </row>
     <row r="36" spans="2:5" x14ac:dyDescent="0.45">
@@ -2784,7 +2778,7 @@
         <v>210</v>
       </c>
       <c r="E36" t="s">
-        <v>147</v>
+        <v>40</v>
       </c>
     </row>
     <row r="37" spans="2:5" x14ac:dyDescent="0.45">
@@ -2798,7 +2792,7 @@
         <v>212</v>
       </c>
       <c r="E37" t="s">
-        <v>147</v>
+        <v>40</v>
       </c>
     </row>
     <row r="38" spans="2:5" x14ac:dyDescent="0.45">
@@ -2812,7 +2806,7 @@
         <v>214</v>
       </c>
       <c r="E38" t="s">
-        <v>147</v>
+        <v>40</v>
       </c>
     </row>
     <row r="39" spans="2:5" x14ac:dyDescent="0.45">
@@ -2826,7 +2820,7 @@
         <v>216</v>
       </c>
       <c r="E39" t="s">
-        <v>147</v>
+        <v>40</v>
       </c>
     </row>
     <row r="40" spans="2:5" x14ac:dyDescent="0.45">
@@ -2840,7 +2834,7 @@
         <v>218</v>
       </c>
       <c r="E40" t="s">
-        <v>147</v>
+        <v>40</v>
       </c>
     </row>
     <row r="41" spans="2:5" x14ac:dyDescent="0.45">
@@ -2854,7 +2848,7 @@
         <v>220</v>
       </c>
       <c r="E41" t="s">
-        <v>147</v>
+        <v>40</v>
       </c>
     </row>
     <row r="42" spans="2:5" x14ac:dyDescent="0.45">
@@ -2868,7 +2862,7 @@
         <v>222</v>
       </c>
       <c r="E42" t="s">
-        <v>147</v>
+        <v>40</v>
       </c>
     </row>
     <row r="43" spans="2:5" x14ac:dyDescent="0.45">
@@ -2882,7 +2876,7 @@
         <v>224</v>
       </c>
       <c r="E43" t="s">
-        <v>147</v>
+        <v>40</v>
       </c>
     </row>
     <row r="44" spans="2:5" x14ac:dyDescent="0.45">
@@ -2896,7 +2890,7 @@
         <v>226</v>
       </c>
       <c r="E44" t="s">
-        <v>147</v>
+        <v>40</v>
       </c>
     </row>
     <row r="45" spans="2:5" x14ac:dyDescent="0.45">
@@ -2910,7 +2904,7 @@
         <v>228</v>
       </c>
       <c r="E45" t="s">
-        <v>147</v>
+        <v>40</v>
       </c>
     </row>
     <row r="46" spans="2:5" x14ac:dyDescent="0.45">
@@ -2924,7 +2918,7 @@
         <v>230</v>
       </c>
       <c r="E46" t="s">
-        <v>147</v>
+        <v>40</v>
       </c>
     </row>
     <row r="47" spans="2:5" x14ac:dyDescent="0.45">
@@ -2938,7 +2932,7 @@
         <v>232</v>
       </c>
       <c r="E47" t="s">
-        <v>147</v>
+        <v>40</v>
       </c>
     </row>
     <row r="48" spans="2:5" x14ac:dyDescent="0.45">
@@ -2952,7 +2946,7 @@
         <v>234</v>
       </c>
       <c r="E48" t="s">
-        <v>147</v>
+        <v>40</v>
       </c>
     </row>
     <row r="49" spans="2:5" x14ac:dyDescent="0.45">
@@ -2966,7 +2960,7 @@
         <v>236</v>
       </c>
       <c r="E49" t="s">
-        <v>147</v>
+        <v>40</v>
       </c>
     </row>
     <row r="50" spans="2:5" x14ac:dyDescent="0.45">
@@ -2980,7 +2974,7 @@
         <v>238</v>
       </c>
       <c r="E50" t="s">
-        <v>147</v>
+        <v>40</v>
       </c>
     </row>
     <row r="51" spans="2:5" x14ac:dyDescent="0.45">
@@ -2994,7 +2988,7 @@
         <v>240</v>
       </c>
       <c r="E51" t="s">
-        <v>147</v>
+        <v>40</v>
       </c>
     </row>
     <row r="52" spans="2:5" x14ac:dyDescent="0.45">
@@ -3008,7 +3002,7 @@
         <v>242</v>
       </c>
       <c r="E52" t="s">
-        <v>147</v>
+        <v>40</v>
       </c>
     </row>
     <row r="53" spans="2:5" x14ac:dyDescent="0.45">
@@ -3022,7 +3016,7 @@
         <v>244</v>
       </c>
       <c r="E53" t="s">
-        <v>147</v>
+        <v>40</v>
       </c>
     </row>
     <row r="54" spans="2:5" x14ac:dyDescent="0.45">
@@ -3036,7 +3030,7 @@
         <v>246</v>
       </c>
       <c r="E54" t="s">
-        <v>147</v>
+        <v>40</v>
       </c>
     </row>
     <row r="55" spans="2:5" x14ac:dyDescent="0.45">
@@ -3050,7 +3044,7 @@
         <v>248</v>
       </c>
       <c r="E55" t="s">
-        <v>147</v>
+        <v>40</v>
       </c>
     </row>
     <row r="56" spans="2:5" x14ac:dyDescent="0.45">
@@ -3064,7 +3058,7 @@
         <v>250</v>
       </c>
       <c r="E56" t="s">
-        <v>147</v>
+        <v>40</v>
       </c>
     </row>
     <row r="57" spans="2:5" x14ac:dyDescent="0.45">
@@ -3078,7 +3072,7 @@
         <v>252</v>
       </c>
       <c r="E57" t="s">
-        <v>147</v>
+        <v>40</v>
       </c>
     </row>
     <row r="58" spans="2:5" x14ac:dyDescent="0.45">
@@ -3092,7 +3086,7 @@
         <v>254</v>
       </c>
       <c r="E58" t="s">
-        <v>147</v>
+        <v>40</v>
       </c>
     </row>
     <row r="59" spans="2:5" x14ac:dyDescent="0.45">
@@ -3106,7 +3100,7 @@
         <v>256</v>
       </c>
       <c r="E59" t="s">
-        <v>147</v>
+        <v>40</v>
       </c>
     </row>
     <row r="60" spans="2:5" x14ac:dyDescent="0.45">
@@ -3120,7 +3114,7 @@
         <v>258</v>
       </c>
       <c r="E60" t="s">
-        <v>147</v>
+        <v>40</v>
       </c>
     </row>
     <row r="61" spans="2:5" x14ac:dyDescent="0.45">
@@ -3134,7 +3128,7 @@
         <v>260</v>
       </c>
       <c r="E61" t="s">
-        <v>147</v>
+        <v>40</v>
       </c>
     </row>
     <row r="62" spans="2:5" x14ac:dyDescent="0.45">
@@ -3148,7 +3142,7 @@
         <v>262</v>
       </c>
       <c r="E62" t="s">
-        <v>147</v>
+        <v>40</v>
       </c>
     </row>
     <row r="63" spans="2:5" x14ac:dyDescent="0.45">
@@ -3162,7 +3156,7 @@
         <v>264</v>
       </c>
       <c r="E63" t="s">
-        <v>147</v>
+        <v>40</v>
       </c>
     </row>
     <row r="64" spans="2:5" x14ac:dyDescent="0.45">
@@ -3176,7 +3170,7 @@
         <v>266</v>
       </c>
       <c r="E64" t="s">
-        <v>147</v>
+        <v>40</v>
       </c>
     </row>
     <row r="65" spans="2:5" x14ac:dyDescent="0.45">
@@ -3190,7 +3184,7 @@
         <v>268</v>
       </c>
       <c r="E65" t="s">
-        <v>147</v>
+        <v>40</v>
       </c>
     </row>
     <row r="66" spans="2:5" x14ac:dyDescent="0.45">
@@ -3204,7 +3198,7 @@
         <v>270</v>
       </c>
       <c r="E66" t="s">
-        <v>147</v>
+        <v>40</v>
       </c>
     </row>
     <row r="67" spans="2:5" x14ac:dyDescent="0.45">
@@ -3218,7 +3212,7 @@
         <v>272</v>
       </c>
       <c r="E67" t="s">
-        <v>147</v>
+        <v>40</v>
       </c>
     </row>
     <row r="68" spans="2:5" x14ac:dyDescent="0.45">
@@ -3232,7 +3226,7 @@
         <v>274</v>
       </c>
       <c r="E68" t="s">
-        <v>147</v>
+        <v>40</v>
       </c>
     </row>
     <row r="69" spans="2:5" x14ac:dyDescent="0.45">
@@ -3246,7 +3240,7 @@
         <v>276</v>
       </c>
       <c r="E69" t="s">
-        <v>147</v>
+        <v>40</v>
       </c>
     </row>
     <row r="70" spans="2:5" x14ac:dyDescent="0.45">
@@ -3260,7 +3254,7 @@
         <v>278</v>
       </c>
       <c r="E70" t="s">
-        <v>147</v>
+        <v>40</v>
       </c>
     </row>
     <row r="71" spans="2:5" x14ac:dyDescent="0.45">
@@ -3274,7 +3268,7 @@
         <v>280</v>
       </c>
       <c r="E71" t="s">
-        <v>147</v>
+        <v>40</v>
       </c>
     </row>
     <row r="72" spans="2:5" x14ac:dyDescent="0.45">
@@ -3288,7 +3282,7 @@
         <v>282</v>
       </c>
       <c r="E72" t="s">
-        <v>147</v>
+        <v>40</v>
       </c>
     </row>
     <row r="73" spans="2:5" x14ac:dyDescent="0.45">
@@ -3302,7 +3296,7 @@
         <v>284</v>
       </c>
       <c r="E73" t="s">
-        <v>147</v>
+        <v>40</v>
       </c>
     </row>
     <row r="74" spans="2:5" x14ac:dyDescent="0.45">
@@ -3316,7 +3310,7 @@
         <v>286</v>
       </c>
       <c r="E74" t="s">
-        <v>147</v>
+        <v>40</v>
       </c>
     </row>
     <row r="75" spans="2:5" x14ac:dyDescent="0.45">
@@ -3330,7 +3324,7 @@
         <v>288</v>
       </c>
       <c r="E75" t="s">
-        <v>147</v>
+        <v>40</v>
       </c>
     </row>
     <row r="76" spans="2:5" x14ac:dyDescent="0.45">
@@ -3344,7 +3338,7 @@
         <v>290</v>
       </c>
       <c r="E76" t="s">
-        <v>147</v>
+        <v>40</v>
       </c>
     </row>
     <row r="77" spans="2:5" x14ac:dyDescent="0.45">
@@ -3358,7 +3352,7 @@
         <v>292</v>
       </c>
       <c r="E77" t="s">
-        <v>147</v>
+        <v>40</v>
       </c>
     </row>
     <row r="78" spans="2:5" x14ac:dyDescent="0.45">
@@ -3372,7 +3366,7 @@
         <v>294</v>
       </c>
       <c r="E78" t="s">
-        <v>147</v>
+        <v>40</v>
       </c>
     </row>
     <row r="79" spans="2:5" x14ac:dyDescent="0.45">
@@ -3386,7 +3380,7 @@
         <v>296</v>
       </c>
       <c r="E79" t="s">
-        <v>147</v>
+        <v>40</v>
       </c>
     </row>
     <row r="80" spans="2:5" x14ac:dyDescent="0.45">
@@ -3400,7 +3394,7 @@
         <v>298</v>
       </c>
       <c r="E80" t="s">
-        <v>147</v>
+        <v>40</v>
       </c>
     </row>
     <row r="81" spans="2:5" x14ac:dyDescent="0.45">
@@ -3414,7 +3408,7 @@
         <v>300</v>
       </c>
       <c r="E81" t="s">
-        <v>147</v>
+        <v>40</v>
       </c>
     </row>
     <row r="82" spans="2:5" x14ac:dyDescent="0.45">
@@ -3428,7 +3422,7 @@
         <v>302</v>
       </c>
       <c r="E82" t="s">
-        <v>147</v>
+        <v>40</v>
       </c>
     </row>
     <row r="83" spans="2:5" x14ac:dyDescent="0.45">
@@ -3442,7 +3436,7 @@
         <v>304</v>
       </c>
       <c r="E83" t="s">
-        <v>147</v>
+        <v>40</v>
       </c>
     </row>
     <row r="84" spans="2:5" x14ac:dyDescent="0.45">
@@ -3456,7 +3450,7 @@
         <v>306</v>
       </c>
       <c r="E84" t="s">
-        <v>147</v>
+        <v>40</v>
       </c>
     </row>
     <row r="85" spans="2:5" x14ac:dyDescent="0.45">
@@ -3470,7 +3464,7 @@
         <v>308</v>
       </c>
       <c r="E85" t="s">
-        <v>147</v>
+        <v>40</v>
       </c>
     </row>
     <row r="86" spans="2:5" x14ac:dyDescent="0.45">
@@ -3484,7 +3478,7 @@
         <v>310</v>
       </c>
       <c r="E86" t="s">
-        <v>147</v>
+        <v>40</v>
       </c>
     </row>
     <row r="87" spans="2:5" x14ac:dyDescent="0.45">
@@ -3498,7 +3492,7 @@
         <v>312</v>
       </c>
       <c r="E87" t="s">
-        <v>147</v>
+        <v>40</v>
       </c>
     </row>
     <row r="88" spans="2:5" x14ac:dyDescent="0.45">
@@ -3512,7 +3506,7 @@
         <v>314</v>
       </c>
       <c r="E88" t="s">
-        <v>147</v>
+        <v>40</v>
       </c>
     </row>
     <row r="89" spans="2:5" x14ac:dyDescent="0.45">
@@ -3526,7 +3520,7 @@
         <v>316</v>
       </c>
       <c r="E89" t="s">
-        <v>147</v>
+        <v>40</v>
       </c>
     </row>
     <row r="90" spans="2:5" x14ac:dyDescent="0.45">
@@ -3540,7 +3534,7 @@
         <v>318</v>
       </c>
       <c r="E90" t="s">
-        <v>147</v>
+        <v>40</v>
       </c>
     </row>
     <row r="91" spans="2:5" x14ac:dyDescent="0.45">
@@ -3554,7 +3548,7 @@
         <v>320</v>
       </c>
       <c r="E91" t="s">
-        <v>147</v>
+        <v>40</v>
       </c>
     </row>
     <row r="92" spans="2:5" x14ac:dyDescent="0.45">
@@ -3568,7 +3562,7 @@
         <v>322</v>
       </c>
       <c r="E92" t="s">
-        <v>147</v>
+        <v>40</v>
       </c>
     </row>
     <row r="93" spans="2:5" x14ac:dyDescent="0.45">
@@ -3582,7 +3576,7 @@
         <v>324</v>
       </c>
       <c r="E93" t="s">
-        <v>147</v>
+        <v>40</v>
       </c>
     </row>
     <row r="94" spans="2:5" x14ac:dyDescent="0.45">
@@ -3596,7 +3590,7 @@
         <v>326</v>
       </c>
       <c r="E94" t="s">
-        <v>147</v>
+        <v>40</v>
       </c>
     </row>
     <row r="95" spans="2:5" x14ac:dyDescent="0.45">
@@ -3610,7 +3604,7 @@
         <v>328</v>
       </c>
       <c r="E95" t="s">
-        <v>147</v>
+        <v>40</v>
       </c>
     </row>
     <row r="96" spans="2:5" x14ac:dyDescent="0.45">
@@ -3624,7 +3618,7 @@
         <v>330</v>
       </c>
       <c r="E96" t="s">
-        <v>147</v>
+        <v>40</v>
       </c>
     </row>
     <row r="97" spans="2:5" x14ac:dyDescent="0.45">
@@ -3638,7 +3632,7 @@
         <v>332</v>
       </c>
       <c r="E97" t="s">
-        <v>147</v>
+        <v>40</v>
       </c>
     </row>
     <row r="98" spans="2:5" x14ac:dyDescent="0.45">
@@ -3652,7 +3646,7 @@
         <v>334</v>
       </c>
       <c r="E98" t="s">
-        <v>147</v>
+        <v>40</v>
       </c>
     </row>
     <row r="99" spans="2:5" x14ac:dyDescent="0.45">
@@ -3666,7 +3660,7 @@
         <v>336</v>
       </c>
       <c r="E99" t="s">
-        <v>147</v>
+        <v>40</v>
       </c>
     </row>
     <row r="100" spans="2:5" x14ac:dyDescent="0.45">
@@ -3680,7 +3674,7 @@
         <v>338</v>
       </c>
       <c r="E100" t="s">
-        <v>147</v>
+        <v>40</v>
       </c>
     </row>
     <row r="101" spans="2:5" x14ac:dyDescent="0.45">
@@ -3694,7 +3688,7 @@
         <v>340</v>
       </c>
       <c r="E101" t="s">
-        <v>147</v>
+        <v>40</v>
       </c>
     </row>
     <row r="102" spans="2:5" x14ac:dyDescent="0.45">
@@ -3708,7 +3702,7 @@
         <v>342</v>
       </c>
       <c r="E102" t="s">
-        <v>147</v>
+        <v>40</v>
       </c>
     </row>
     <row r="103" spans="2:5" x14ac:dyDescent="0.45">
@@ -3722,7 +3716,7 @@
         <v>344</v>
       </c>
       <c r="E103" t="s">
-        <v>147</v>
+        <v>40</v>
       </c>
     </row>
     <row r="104" spans="2:5" x14ac:dyDescent="0.45">
@@ -3736,7 +3730,7 @@
         <v>346</v>
       </c>
       <c r="E104" t="s">
-        <v>147</v>
+        <v>40</v>
       </c>
     </row>
     <row r="105" spans="2:5" x14ac:dyDescent="0.45">
@@ -3750,7 +3744,7 @@
         <v>348</v>
       </c>
       <c r="E105" t="s">
-        <v>147</v>
+        <v>40</v>
       </c>
     </row>
     <row r="106" spans="2:5" x14ac:dyDescent="0.45">
@@ -3764,7 +3758,7 @@
         <v>350</v>
       </c>
       <c r="E106" t="s">
-        <v>147</v>
+        <v>40</v>
       </c>
     </row>
     <row r="107" spans="2:5" x14ac:dyDescent="0.45">
@@ -3778,7 +3772,7 @@
         <v>352</v>
       </c>
       <c r="E107" t="s">
-        <v>147</v>
+        <v>40</v>
       </c>
     </row>
     <row r="108" spans="2:5" x14ac:dyDescent="0.45">
@@ -3792,7 +3786,7 @@
         <v>354</v>
       </c>
       <c r="E108" t="s">
-        <v>147</v>
+        <v>40</v>
       </c>
     </row>
     <row r="109" spans="2:5" x14ac:dyDescent="0.45">
@@ -3806,7 +3800,7 @@
         <v>356</v>
       </c>
       <c r="E109" t="s">
-        <v>147</v>
+        <v>40</v>
       </c>
     </row>
     <row r="110" spans="2:5" x14ac:dyDescent="0.45">
@@ -3820,7 +3814,7 @@
         <v>358</v>
       </c>
       <c r="E110" t="s">
-        <v>147</v>
+        <v>40</v>
       </c>
     </row>
     <row r="111" spans="2:5" x14ac:dyDescent="0.45">
@@ -3834,7 +3828,7 @@
         <v>360</v>
       </c>
       <c r="E111" t="s">
-        <v>147</v>
+        <v>40</v>
       </c>
     </row>
     <row r="112" spans="2:5" x14ac:dyDescent="0.45">
@@ -3848,7 +3842,7 @@
         <v>362</v>
       </c>
       <c r="E112" t="s">
-        <v>147</v>
+        <v>40</v>
       </c>
     </row>
     <row r="113" spans="2:5" x14ac:dyDescent="0.45">
@@ -3862,7 +3856,7 @@
         <v>364</v>
       </c>
       <c r="E113" t="s">
-        <v>147</v>
+        <v>40</v>
       </c>
     </row>
     <row r="114" spans="2:5" x14ac:dyDescent="0.45">
@@ -3876,7 +3870,7 @@
         <v>366</v>
       </c>
       <c r="E114" t="s">
-        <v>147</v>
+        <v>40</v>
       </c>
     </row>
     <row r="115" spans="2:5" x14ac:dyDescent="0.45">
@@ -3890,7 +3884,7 @@
         <v>368</v>
       </c>
       <c r="E115" t="s">
-        <v>147</v>
+        <v>40</v>
       </c>
     </row>
     <row r="116" spans="2:5" x14ac:dyDescent="0.45">
@@ -3904,7 +3898,7 @@
         <v>370</v>
       </c>
       <c r="E116" t="s">
-        <v>147</v>
+        <v>40</v>
       </c>
     </row>
     <row r="117" spans="2:5" x14ac:dyDescent="0.45">
@@ -3918,7 +3912,7 @@
         <v>372</v>
       </c>
       <c r="E117" t="s">
-        <v>147</v>
+        <v>40</v>
       </c>
     </row>
     <row r="118" spans="2:5" x14ac:dyDescent="0.45">
@@ -3932,7 +3926,7 @@
         <v>374</v>
       </c>
       <c r="E118" t="s">
-        <v>147</v>
+        <v>40</v>
       </c>
     </row>
     <row r="119" spans="2:5" x14ac:dyDescent="0.45">
@@ -3946,7 +3940,7 @@
         <v>376</v>
       </c>
       <c r="E119" t="s">
-        <v>147</v>
+        <v>40</v>
       </c>
     </row>
     <row r="120" spans="2:5" x14ac:dyDescent="0.45">
@@ -3960,7 +3954,7 @@
         <v>378</v>
       </c>
       <c r="E120" t="s">
-        <v>147</v>
+        <v>40</v>
       </c>
     </row>
     <row r="121" spans="2:5" x14ac:dyDescent="0.45">
@@ -3974,7 +3968,7 @@
         <v>380</v>
       </c>
       <c r="E121" t="s">
-        <v>147</v>
+        <v>40</v>
       </c>
     </row>
     <row r="122" spans="2:5" x14ac:dyDescent="0.45">
@@ -3988,7 +3982,7 @@
         <v>382</v>
       </c>
       <c r="E122" t="s">
-        <v>147</v>
+        <v>40</v>
       </c>
     </row>
     <row r="123" spans="2:5" x14ac:dyDescent="0.45">
@@ -4002,7 +3996,7 @@
         <v>384</v>
       </c>
       <c r="E123" t="s">
-        <v>147</v>
+        <v>40</v>
       </c>
     </row>
     <row r="124" spans="2:5" x14ac:dyDescent="0.45">
@@ -4016,7 +4010,7 @@
         <v>386</v>
       </c>
       <c r="E124" t="s">
-        <v>147</v>
+        <v>40</v>
       </c>
     </row>
     <row r="125" spans="2:5" x14ac:dyDescent="0.45">
@@ -4030,7 +4024,7 @@
         <v>388</v>
       </c>
       <c r="E125" t="s">
-        <v>147</v>
+        <v>40</v>
       </c>
     </row>
     <row r="126" spans="2:5" x14ac:dyDescent="0.45">
@@ -4044,7 +4038,7 @@
         <v>390</v>
       </c>
       <c r="E126" t="s">
-        <v>147</v>
+        <v>40</v>
       </c>
     </row>
     <row r="127" spans="2:5" x14ac:dyDescent="0.45">
@@ -4058,7 +4052,7 @@
         <v>392</v>
       </c>
       <c r="E127" t="s">
-        <v>147</v>
+        <v>40</v>
       </c>
     </row>
     <row r="128" spans="2:5" x14ac:dyDescent="0.45">
@@ -4072,7 +4066,7 @@
         <v>394</v>
       </c>
       <c r="E128" t="s">
-        <v>147</v>
+        <v>40</v>
       </c>
     </row>
     <row r="129" spans="2:5" x14ac:dyDescent="0.45">
@@ -4086,7 +4080,7 @@
         <v>396</v>
       </c>
       <c r="E129" t="s">
-        <v>147</v>
+        <v>40</v>
       </c>
     </row>
     <row r="130" spans="2:5" x14ac:dyDescent="0.45">
@@ -4100,7 +4094,7 @@
         <v>398</v>
       </c>
       <c r="E130" t="s">
-        <v>147</v>
+        <v>40</v>
       </c>
     </row>
     <row r="131" spans="2:5" x14ac:dyDescent="0.45">
@@ -4114,7 +4108,7 @@
         <v>400</v>
       </c>
       <c r="E131" t="s">
-        <v>147</v>
+        <v>40</v>
       </c>
     </row>
     <row r="132" spans="2:5" x14ac:dyDescent="0.45">
@@ -4128,7 +4122,7 @@
         <v>402</v>
       </c>
       <c r="E132" t="s">
-        <v>147</v>
+        <v>40</v>
       </c>
     </row>
     <row r="133" spans="2:5" x14ac:dyDescent="0.45">
@@ -4142,7 +4136,7 @@
         <v>404</v>
       </c>
       <c r="E133" t="s">
-        <v>147</v>
+        <v>40</v>
       </c>
     </row>
     <row r="134" spans="2:5" x14ac:dyDescent="0.45">
@@ -4156,7 +4150,7 @@
         <v>406</v>
       </c>
       <c r="E134" t="s">
-        <v>147</v>
+        <v>40</v>
       </c>
     </row>
     <row r="135" spans="2:5" x14ac:dyDescent="0.45">
@@ -4170,7 +4164,7 @@
         <v>408</v>
       </c>
       <c r="E135" t="s">
-        <v>147</v>
+        <v>40</v>
       </c>
     </row>
     <row r="136" spans="2:5" x14ac:dyDescent="0.45">
@@ -4184,7 +4178,7 @@
         <v>410</v>
       </c>
       <c r="E136" t="s">
-        <v>147</v>
+        <v>40</v>
       </c>
     </row>
     <row r="137" spans="2:5" x14ac:dyDescent="0.45">
@@ -4198,7 +4192,7 @@
         <v>412</v>
       </c>
       <c r="E137" t="s">
-        <v>147</v>
+        <v>40</v>
       </c>
     </row>
     <row r="138" spans="2:5" x14ac:dyDescent="0.45">
@@ -4212,7 +4206,7 @@
         <v>414</v>
       </c>
       <c r="E138" t="s">
-        <v>147</v>
+        <v>40</v>
       </c>
     </row>
     <row r="139" spans="2:5" x14ac:dyDescent="0.45">
@@ -4226,7 +4220,7 @@
         <v>416</v>
       </c>
       <c r="E139" t="s">
-        <v>147</v>
+        <v>40</v>
       </c>
     </row>
     <row r="140" spans="2:5" x14ac:dyDescent="0.45">
@@ -4240,7 +4234,7 @@
         <v>418</v>
       </c>
       <c r="E140" t="s">
-        <v>147</v>
+        <v>40</v>
       </c>
     </row>
     <row r="141" spans="2:5" x14ac:dyDescent="0.45">
@@ -4254,7 +4248,7 @@
         <v>420</v>
       </c>
       <c r="E141" t="s">
-        <v>147</v>
+        <v>40</v>
       </c>
     </row>
     <row r="142" spans="2:5" x14ac:dyDescent="0.45">
@@ -4268,7 +4262,7 @@
         <v>422</v>
       </c>
       <c r="E142" t="s">
-        <v>147</v>
+        <v>40</v>
       </c>
     </row>
     <row r="143" spans="2:5" x14ac:dyDescent="0.45">
@@ -4282,7 +4276,7 @@
         <v>424</v>
       </c>
       <c r="E143" t="s">
-        <v>147</v>
+        <v>40</v>
       </c>
     </row>
     <row r="144" spans="2:5" x14ac:dyDescent="0.45">
@@ -4296,7 +4290,7 @@
         <v>426</v>
       </c>
       <c r="E144" t="s">
-        <v>147</v>
+        <v>40</v>
       </c>
     </row>
     <row r="145" spans="2:5" x14ac:dyDescent="0.45">
@@ -4310,7 +4304,7 @@
         <v>428</v>
       </c>
       <c r="E145" t="s">
-        <v>147</v>
+        <v>40</v>
       </c>
     </row>
     <row r="146" spans="2:5" x14ac:dyDescent="0.45">
@@ -4324,7 +4318,7 @@
         <v>430</v>
       </c>
       <c r="E146" t="s">
-        <v>147</v>
+        <v>40</v>
       </c>
     </row>
     <row r="147" spans="2:5" x14ac:dyDescent="0.45">
@@ -4338,7 +4332,7 @@
         <v>432</v>
       </c>
       <c r="E147" t="s">
-        <v>147</v>
+        <v>40</v>
       </c>
     </row>
     <row r="148" spans="2:5" x14ac:dyDescent="0.45">
@@ -4352,7 +4346,7 @@
         <v>434</v>
       </c>
       <c r="E148" t="s">
-        <v>147</v>
+        <v>40</v>
       </c>
     </row>
     <row r="149" spans="2:5" x14ac:dyDescent="0.45">
@@ -4366,7 +4360,7 @@
         <v>436</v>
       </c>
       <c r="E149" t="s">
-        <v>147</v>
+        <v>40</v>
       </c>
     </row>
     <row r="150" spans="2:5" x14ac:dyDescent="0.45">
@@ -4380,7 +4374,7 @@
         <v>438</v>
       </c>
       <c r="E150" t="s">
-        <v>147</v>
+        <v>40</v>
       </c>
     </row>
     <row r="151" spans="2:5" x14ac:dyDescent="0.45">
@@ -4394,7 +4388,7 @@
         <v>440</v>
       </c>
       <c r="E151" t="s">
-        <v>147</v>
+        <v>40</v>
       </c>
     </row>
     <row r="152" spans="2:5" x14ac:dyDescent="0.45">
@@ -4408,7 +4402,7 @@
         <v>442</v>
       </c>
       <c r="E152" t="s">
-        <v>147</v>
+        <v>40</v>
       </c>
     </row>
     <row r="153" spans="2:5" x14ac:dyDescent="0.45">
@@ -4422,7 +4416,7 @@
         <v>444</v>
       </c>
       <c r="E153" t="s">
-        <v>147</v>
+        <v>40</v>
       </c>
     </row>
     <row r="154" spans="2:5" x14ac:dyDescent="0.45">
@@ -4436,7 +4430,7 @@
         <v>446</v>
       </c>
       <c r="E154" t="s">
-        <v>147</v>
+        <v>40</v>
       </c>
     </row>
     <row r="155" spans="2:5" x14ac:dyDescent="0.45">
@@ -4450,7 +4444,7 @@
         <v>448</v>
       </c>
       <c r="E155" t="s">
-        <v>147</v>
+        <v>40</v>
       </c>
     </row>
     <row r="156" spans="2:5" x14ac:dyDescent="0.45">
@@ -4464,7 +4458,7 @@
         <v>450</v>
       </c>
       <c r="E156" t="s">
-        <v>147</v>
+        <v>40</v>
       </c>
     </row>
     <row r="157" spans="2:5" x14ac:dyDescent="0.45">
@@ -4478,7 +4472,7 @@
         <v>452</v>
       </c>
       <c r="E157" t="s">
-        <v>147</v>
+        <v>40</v>
       </c>
     </row>
     <row r="158" spans="2:5" x14ac:dyDescent="0.45">
@@ -4492,7 +4486,7 @@
         <v>454</v>
       </c>
       <c r="E158" t="s">
-        <v>147</v>
+        <v>40</v>
       </c>
     </row>
     <row r="159" spans="2:5" x14ac:dyDescent="0.45">
@@ -4506,7 +4500,7 @@
         <v>456</v>
       </c>
       <c r="E159" t="s">
-        <v>147</v>
+        <v>40</v>
       </c>
     </row>
     <row r="160" spans="2:5" x14ac:dyDescent="0.45">
@@ -4520,7 +4514,7 @@
         <v>458</v>
       </c>
       <c r="E160" t="s">
-        <v>147</v>
+        <v>40</v>
       </c>
     </row>
     <row r="161" spans="2:5" x14ac:dyDescent="0.45">
@@ -4534,7 +4528,7 @@
         <v>460</v>
       </c>
       <c r="E161" t="s">
-        <v>147</v>
+        <v>40</v>
       </c>
     </row>
     <row r="162" spans="2:5" x14ac:dyDescent="0.45">
@@ -4548,7 +4542,7 @@
         <v>462</v>
       </c>
       <c r="E162" t="s">
-        <v>147</v>
+        <v>40</v>
       </c>
     </row>
     <row r="163" spans="2:5" x14ac:dyDescent="0.45">
@@ -4562,7 +4556,7 @@
         <v>464</v>
       </c>
       <c r="E163" t="s">
-        <v>147</v>
+        <v>40</v>
       </c>
     </row>
     <row r="164" spans="2:5" x14ac:dyDescent="0.45">
@@ -4576,7 +4570,7 @@
         <v>466</v>
       </c>
       <c r="E164" t="s">
-        <v>147</v>
+        <v>40</v>
       </c>
     </row>
     <row r="165" spans="2:5" x14ac:dyDescent="0.45">
@@ -4590,7 +4584,7 @@
         <v>468</v>
       </c>
       <c r="E165" t="s">
-        <v>147</v>
+        <v>40</v>
       </c>
     </row>
     <row r="166" spans="2:5" x14ac:dyDescent="0.45">
@@ -4604,7 +4598,7 @@
         <v>470</v>
       </c>
       <c r="E166" t="s">
-        <v>147</v>
+        <v>40</v>
       </c>
     </row>
     <row r="167" spans="2:5" x14ac:dyDescent="0.45">
@@ -4618,7 +4612,7 @@
         <v>472</v>
       </c>
       <c r="E167" t="s">
-        <v>147</v>
+        <v>40</v>
       </c>
     </row>
     <row r="168" spans="2:5" x14ac:dyDescent="0.45">
@@ -4632,7 +4626,7 @@
         <v>474</v>
       </c>
       <c r="E168" t="s">
-        <v>147</v>
+        <v>40</v>
       </c>
     </row>
     <row r="169" spans="2:5" x14ac:dyDescent="0.45">
@@ -4646,7 +4640,7 @@
         <v>476</v>
       </c>
       <c r="E169" t="s">
-        <v>147</v>
+        <v>40</v>
       </c>
     </row>
     <row r="170" spans="2:5" x14ac:dyDescent="0.45">
@@ -4660,7 +4654,7 @@
         <v>478</v>
       </c>
       <c r="E170" t="s">
-        <v>147</v>
+        <v>40</v>
       </c>
     </row>
     <row r="171" spans="2:5" x14ac:dyDescent="0.45">
@@ -4674,7 +4668,7 @@
         <v>480</v>
       </c>
       <c r="E171" t="s">
-        <v>147</v>
+        <v>40</v>
       </c>
     </row>
     <row r="172" spans="2:5" x14ac:dyDescent="0.45">
@@ -4688,7 +4682,7 @@
         <v>482</v>
       </c>
       <c r="E172" t="s">
-        <v>147</v>
+        <v>40</v>
       </c>
     </row>
     <row r="173" spans="2:5" x14ac:dyDescent="0.45">
@@ -4702,7 +4696,7 @@
         <v>484</v>
       </c>
       <c r="E173" t="s">
-        <v>147</v>
+        <v>40</v>
       </c>
     </row>
     <row r="174" spans="2:5" x14ac:dyDescent="0.45">
@@ -4716,7 +4710,7 @@
         <v>486</v>
       </c>
       <c r="E174" t="s">
-        <v>147</v>
+        <v>40</v>
       </c>
     </row>
     <row r="175" spans="2:5" x14ac:dyDescent="0.45">
@@ -4730,7 +4724,7 @@
         <v>488</v>
       </c>
       <c r="E175" t="s">
-        <v>147</v>
+        <v>40</v>
       </c>
     </row>
     <row r="176" spans="2:5" x14ac:dyDescent="0.45">
@@ -4744,7 +4738,7 @@
         <v>490</v>
       </c>
       <c r="E176" t="s">
-        <v>147</v>
+        <v>40</v>
       </c>
     </row>
     <row r="177" spans="2:5" x14ac:dyDescent="0.45">
@@ -4758,7 +4752,7 @@
         <v>492</v>
       </c>
       <c r="E177" t="s">
-        <v>147</v>
+        <v>40</v>
       </c>
     </row>
     <row r="178" spans="2:5" x14ac:dyDescent="0.45">
@@ -4772,7 +4766,7 @@
         <v>494</v>
       </c>
       <c r="E178" t="s">
-        <v>147</v>
+        <v>40</v>
       </c>
     </row>
     <row r="179" spans="2:5" x14ac:dyDescent="0.45">
@@ -4786,7 +4780,7 @@
         <v>496</v>
       </c>
       <c r="E179" t="s">
-        <v>147</v>
+        <v>40</v>
       </c>
     </row>
     <row r="180" spans="2:5" x14ac:dyDescent="0.45">
@@ -4800,7 +4794,7 @@
         <v>498</v>
       </c>
       <c r="E180" t="s">
-        <v>147</v>
+        <v>40</v>
       </c>
     </row>
     <row r="181" spans="2:5" x14ac:dyDescent="0.45">
@@ -4814,7 +4808,7 @@
         <v>500</v>
       </c>
       <c r="E181" t="s">
-        <v>147</v>
+        <v>40</v>
       </c>
     </row>
     <row r="182" spans="2:5" x14ac:dyDescent="0.45">
@@ -4828,7 +4822,7 @@
         <v>502</v>
       </c>
       <c r="E182" t="s">
-        <v>147</v>
+        <v>40</v>
       </c>
     </row>
     <row r="183" spans="2:5" x14ac:dyDescent="0.45">
@@ -4842,7 +4836,7 @@
         <v>504</v>
       </c>
       <c r="E183" t="s">
-        <v>147</v>
+        <v>40</v>
       </c>
     </row>
     <row r="184" spans="2:5" x14ac:dyDescent="0.45">
@@ -4856,7 +4850,7 @@
         <v>506</v>
       </c>
       <c r="E184" t="s">
-        <v>147</v>
+        <v>40</v>
       </c>
     </row>
     <row r="185" spans="2:5" x14ac:dyDescent="0.45">
@@ -4870,7 +4864,7 @@
         <v>508</v>
       </c>
       <c r="E185" t="s">
-        <v>147</v>
+        <v>40</v>
       </c>
     </row>
     <row r="186" spans="2:5" x14ac:dyDescent="0.45">
@@ -4884,7 +4878,7 @@
         <v>510</v>
       </c>
       <c r="E186" t="s">
-        <v>147</v>
+        <v>40</v>
       </c>
     </row>
     <row r="187" spans="2:5" x14ac:dyDescent="0.45">
@@ -4898,7 +4892,7 @@
         <v>512</v>
       </c>
       <c r="E187" t="s">
-        <v>147</v>
+        <v>40</v>
       </c>
     </row>
     <row r="188" spans="2:5" x14ac:dyDescent="0.45">
@@ -4912,7 +4906,7 @@
         <v>514</v>
       </c>
       <c r="E188" t="s">
-        <v>147</v>
+        <v>40</v>
       </c>
     </row>
     <row r="189" spans="2:5" x14ac:dyDescent="0.45">
@@ -4926,7 +4920,7 @@
         <v>516</v>
       </c>
       <c r="E189" t="s">
-        <v>147</v>
+        <v>40</v>
       </c>
     </row>
     <row r="190" spans="2:5" x14ac:dyDescent="0.45">
@@ -4940,7 +4934,7 @@
         <v>518</v>
       </c>
       <c r="E190" t="s">
-        <v>147</v>
+        <v>40</v>
       </c>
     </row>
     <row r="191" spans="2:5" x14ac:dyDescent="0.45">
@@ -4954,7 +4948,7 @@
         <v>520</v>
       </c>
       <c r="E191" t="s">
-        <v>147</v>
+        <v>40</v>
       </c>
     </row>
     <row r="192" spans="2:5" x14ac:dyDescent="0.45">
@@ -4968,7 +4962,7 @@
         <v>522</v>
       </c>
       <c r="E192" t="s">
-        <v>147</v>
+        <v>40</v>
       </c>
     </row>
     <row r="193" spans="2:5" x14ac:dyDescent="0.45">
@@ -4982,7 +4976,7 @@
         <v>524</v>
       </c>
       <c r="E193" t="s">
-        <v>147</v>
+        <v>40</v>
       </c>
     </row>
     <row r="194" spans="2:5" x14ac:dyDescent="0.45">
@@ -4996,7 +4990,7 @@
         <v>526</v>
       </c>
       <c r="E194" t="s">
-        <v>147</v>
+        <v>40</v>
       </c>
     </row>
     <row r="195" spans="2:5" x14ac:dyDescent="0.45">
@@ -5010,7 +5004,7 @@
         <v>528</v>
       </c>
       <c r="E195" t="s">
-        <v>147</v>
+        <v>40</v>
       </c>
     </row>
     <row r="196" spans="2:5" x14ac:dyDescent="0.45">
@@ -5024,7 +5018,7 @@
         <v>530</v>
       </c>
       <c r="E196" t="s">
-        <v>147</v>
+        <v>40</v>
       </c>
     </row>
     <row r="197" spans="2:5" x14ac:dyDescent="0.45">
@@ -5038,7 +5032,7 @@
         <v>532</v>
       </c>
       <c r="E197" t="s">
-        <v>147</v>
+        <v>40</v>
       </c>
     </row>
     <row r="198" spans="2:5" x14ac:dyDescent="0.45">
@@ -5052,7 +5046,7 @@
         <v>534</v>
       </c>
       <c r="E198" t="s">
-        <v>147</v>
+        <v>40</v>
       </c>
     </row>
     <row r="199" spans="2:5" x14ac:dyDescent="0.45">
@@ -5066,7 +5060,7 @@
         <v>536</v>
       </c>
       <c r="E199" t="s">
-        <v>147</v>
+        <v>40</v>
       </c>
     </row>
     <row r="200" spans="2:5" x14ac:dyDescent="0.45">
@@ -5080,7 +5074,7 @@
         <v>538</v>
       </c>
       <c r="E200" t="s">
-        <v>147</v>
+        <v>40</v>
       </c>
     </row>
     <row r="201" spans="2:5" x14ac:dyDescent="0.45">
@@ -5094,7 +5088,7 @@
         <v>540</v>
       </c>
       <c r="E201" t="s">
-        <v>147</v>
+        <v>40</v>
       </c>
     </row>
     <row r="202" spans="2:5" x14ac:dyDescent="0.45">
@@ -5108,7 +5102,7 @@
         <v>542</v>
       </c>
       <c r="E202" t="s">
-        <v>147</v>
+        <v>40</v>
       </c>
     </row>
     <row r="203" spans="2:5" x14ac:dyDescent="0.45">
@@ -5122,7 +5116,7 @@
         <v>544</v>
       </c>
       <c r="E203" t="s">
-        <v>147</v>
+        <v>40</v>
       </c>
     </row>
     <row r="204" spans="2:5" x14ac:dyDescent="0.45">
@@ -5136,7 +5130,7 @@
         <v>546</v>
       </c>
       <c r="E204" t="s">
-        <v>147</v>
+        <v>40</v>
       </c>
     </row>
     <row r="205" spans="2:5" x14ac:dyDescent="0.45">
@@ -5150,7 +5144,7 @@
         <v>548</v>
       </c>
       <c r="E205" t="s">
-        <v>147</v>
+        <v>40</v>
       </c>
     </row>
     <row r="206" spans="2:5" x14ac:dyDescent="0.45">
@@ -5164,7 +5158,7 @@
         <v>550</v>
       </c>
       <c r="E206" t="s">
-        <v>147</v>
+        <v>40</v>
       </c>
     </row>
     <row r="207" spans="2:5" x14ac:dyDescent="0.45">
@@ -5178,7 +5172,7 @@
         <v>552</v>
       </c>
       <c r="E207" t="s">
-        <v>147</v>
+        <v>40</v>
       </c>
     </row>
     <row r="208" spans="2:5" x14ac:dyDescent="0.45">
@@ -5192,7 +5186,7 @@
         <v>554</v>
       </c>
       <c r="E208" t="s">
-        <v>147</v>
+        <v>40</v>
       </c>
     </row>
     <row r="209" spans="2:5" x14ac:dyDescent="0.45">
@@ -5206,7 +5200,7 @@
         <v>556</v>
       </c>
       <c r="E209" t="s">
-        <v>147</v>
+        <v>40</v>
       </c>
     </row>
     <row r="210" spans="2:5" x14ac:dyDescent="0.45">
@@ -5220,7 +5214,7 @@
         <v>558</v>
       </c>
       <c r="E210" t="s">
-        <v>147</v>
+        <v>40</v>
       </c>
     </row>
     <row r="211" spans="2:5" x14ac:dyDescent="0.45">
@@ -5234,7 +5228,7 @@
         <v>560</v>
       </c>
       <c r="E211" t="s">
-        <v>147</v>
+        <v>40</v>
       </c>
     </row>
     <row r="212" spans="2:5" x14ac:dyDescent="0.45">
@@ -5248,7 +5242,7 @@
         <v>562</v>
       </c>
       <c r="E212" t="s">
-        <v>147</v>
+        <v>40</v>
       </c>
     </row>
     <row r="213" spans="2:5" x14ac:dyDescent="0.45">
@@ -5262,7 +5256,7 @@
         <v>564</v>
       </c>
       <c r="E213" t="s">
-        <v>147</v>
+        <v>40</v>
       </c>
     </row>
     <row r="214" spans="2:5" x14ac:dyDescent="0.45">
@@ -5276,7 +5270,7 @@
         <v>566</v>
       </c>
       <c r="E214" t="s">
-        <v>147</v>
+        <v>40</v>
       </c>
     </row>
     <row r="215" spans="2:5" x14ac:dyDescent="0.45">
@@ -5290,7 +5284,7 @@
         <v>568</v>
       </c>
       <c r="E215" t="s">
-        <v>147</v>
+        <v>40</v>
       </c>
     </row>
     <row r="216" spans="2:5" x14ac:dyDescent="0.45">
@@ -5304,7 +5298,7 @@
         <v>570</v>
       </c>
       <c r="E216" t="s">
-        <v>147</v>
+        <v>40</v>
       </c>
     </row>
     <row r="217" spans="2:5" x14ac:dyDescent="0.45">
@@ -5318,7 +5312,7 @@
         <v>572</v>
       </c>
       <c r="E217" t="s">
-        <v>147</v>
+        <v>40</v>
       </c>
     </row>
     <row r="218" spans="2:5" x14ac:dyDescent="0.45">
@@ -5332,7 +5326,7 @@
         <v>574</v>
       </c>
       <c r="E218" t="s">
-        <v>147</v>
+        <v>40</v>
       </c>
     </row>
     <row r="219" spans="2:5" x14ac:dyDescent="0.45">
@@ -5346,7 +5340,7 @@
         <v>576</v>
       </c>
       <c r="E219" t="s">
-        <v>147</v>
+        <v>40</v>
       </c>
     </row>
     <row r="220" spans="2:5" x14ac:dyDescent="0.45">
@@ -5360,7 +5354,7 @@
         <v>578</v>
       </c>
       <c r="E220" t="s">
-        <v>147</v>
+        <v>40</v>
       </c>
     </row>
     <row r="221" spans="2:5" x14ac:dyDescent="0.45">
@@ -5374,7 +5368,7 @@
         <v>580</v>
       </c>
       <c r="E221" t="s">
-        <v>147</v>
+        <v>40</v>
       </c>
     </row>
     <row r="222" spans="2:5" x14ac:dyDescent="0.45">
@@ -5388,7 +5382,7 @@
         <v>582</v>
       </c>
       <c r="E222" t="s">
-        <v>147</v>
+        <v>40</v>
       </c>
     </row>
     <row r="223" spans="2:5" x14ac:dyDescent="0.45">
@@ -5402,7 +5396,7 @@
         <v>584</v>
       </c>
       <c r="E223" t="s">
-        <v>147</v>
+        <v>40</v>
       </c>
     </row>
     <row r="224" spans="2:5" x14ac:dyDescent="0.45">
@@ -5416,7 +5410,7 @@
         <v>586</v>
       </c>
       <c r="E224" t="s">
-        <v>147</v>
+        <v>40</v>
       </c>
     </row>
     <row r="225" spans="2:5" x14ac:dyDescent="0.45">
@@ -5430,7 +5424,7 @@
         <v>588</v>
       </c>
       <c r="E225" t="s">
-        <v>147</v>
+        <v>40</v>
       </c>
     </row>
     <row r="226" spans="2:5" x14ac:dyDescent="0.45">
@@ -5444,7 +5438,7 @@
         <v>590</v>
       </c>
       <c r="E226" t="s">
-        <v>147</v>
+        <v>40</v>
       </c>
     </row>
     <row r="227" spans="2:5" x14ac:dyDescent="0.45">
@@ -5458,7 +5452,7 @@
         <v>592</v>
       </c>
       <c r="E227" t="s">
-        <v>147</v>
+        <v>40</v>
       </c>
     </row>
     <row r="228" spans="2:5" x14ac:dyDescent="0.45">
@@ -5472,7 +5466,7 @@
         <v>594</v>
       </c>
       <c r="E228" t="s">
-        <v>147</v>
+        <v>40</v>
       </c>
     </row>
   </sheetData>
@@ -5481,7 +5475,7 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{718D7FD7-C83A-40FD-B4D1-09885A1486FD}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:J47"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
@@ -5497,561 +5491,561 @@
     <col min="10" max="10" width="24.86328125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" ht="17.25" thickBot="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="1" spans="1:10" ht="17.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A1" s="1" t="s">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="2" spans="1:10" ht="15" thickTop="1" thickBot="1" x14ac:dyDescent="0.5">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="2" spans="1:10" ht="15" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.5">
       <c r="A2" s="2" t="s">
-        <v>1</v>
+        <v>42</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>2</v>
+        <v>43</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>3</v>
+        <v>44</v>
       </c>
       <c r="D2" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="E2" s="2" t="s">
+        <v>46</v>
+      </c>
+      <c r="F2" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="E2" s="2" t="s">
+      <c r="G2" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="F2" s="2" t="s">
-        <v>6</v>
-      </c>
-      <c r="G2" s="2" t="s">
-        <v>7</v>
-      </c>
       <c r="H2" s="2" t="s">
+        <v>47</v>
+      </c>
+      <c r="I2" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="J2" s="2" t="s">
         <v>8</v>
-      </c>
-      <c r="I2" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="J2" s="2" t="s">
-        <v>10</v>
       </c>
     </row>
     <row r="3" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A3" t="s">
-        <v>11</v>
+        <v>49</v>
       </c>
       <c r="B3" t="s">
-        <v>157</v>
+        <v>50</v>
       </c>
       <c r="D3" t="s">
-        <v>151</v>
+        <v>51</v>
       </c>
       <c r="F3" t="s">
-        <v>18</v>
+        <v>52</v>
       </c>
       <c r="G3" t="s">
-        <v>72</v>
+        <v>53</v>
       </c>
       <c r="J3" t="s">
-        <v>73</v>
+        <v>54</v>
       </c>
     </row>
     <row r="4" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A4" t="s">
-        <v>11</v>
+        <v>49</v>
       </c>
       <c r="B4" t="s">
-        <v>133</v>
+        <v>55</v>
       </c>
       <c r="D4" t="s">
-        <v>151</v>
+        <v>51</v>
       </c>
       <c r="F4" t="s">
-        <v>74</v>
+        <v>56</v>
       </c>
       <c r="G4" t="s">
-        <v>75</v>
+        <v>57</v>
       </c>
       <c r="J4" t="s">
-        <v>76</v>
+        <v>58</v>
       </c>
     </row>
     <row r="5" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A5" t="s">
-        <v>11</v>
+        <v>49</v>
       </c>
       <c r="B5" t="s">
-        <v>158</v>
+        <v>59</v>
       </c>
       <c r="D5" t="s">
-        <v>151</v>
+        <v>51</v>
       </c>
       <c r="F5" t="s">
-        <v>77</v>
+        <v>60</v>
       </c>
       <c r="G5" t="s">
-        <v>78</v>
+        <v>61</v>
       </c>
     </row>
     <row r="6" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A6" t="s">
-        <v>11</v>
+        <v>49</v>
       </c>
       <c r="B6" t="s">
-        <v>156</v>
+        <v>62</v>
       </c>
       <c r="F6" t="s">
-        <v>79</v>
+        <v>63</v>
       </c>
       <c r="G6" t="s">
-        <v>80</v>
+        <v>64</v>
       </c>
     </row>
     <row r="7" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A7" t="s">
-        <v>11</v>
+        <v>49</v>
       </c>
       <c r="B7" t="s">
-        <v>134</v>
+        <v>65</v>
       </c>
       <c r="D7" t="s">
-        <v>150</v>
+        <v>66</v>
       </c>
       <c r="F7" t="s">
-        <v>81</v>
+        <v>67</v>
       </c>
       <c r="G7" t="s">
-        <v>19</v>
+        <v>68</v>
       </c>
       <c r="J7" t="s">
-        <v>82</v>
+        <v>69</v>
       </c>
     </row>
     <row r="8" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A8" t="s">
-        <v>11</v>
+        <v>49</v>
       </c>
       <c r="B8" t="s">
-        <v>149</v>
+        <v>70</v>
       </c>
       <c r="D8" t="s">
-        <v>150</v>
+        <v>66</v>
       </c>
       <c r="F8" t="s">
-        <v>83</v>
+        <v>71</v>
       </c>
       <c r="G8" t="s">
-        <v>84</v>
+        <v>72</v>
       </c>
       <c r="J8" t="s">
-        <v>85</v>
+        <v>73</v>
       </c>
     </row>
     <row r="9" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A9" t="s">
-        <v>11</v>
+        <v>49</v>
       </c>
       <c r="B9" t="s">
-        <v>86</v>
+        <v>74</v>
       </c>
       <c r="F9" t="s">
-        <v>21</v>
+        <v>75</v>
       </c>
       <c r="G9" t="s">
-        <v>87</v>
+        <v>76</v>
       </c>
     </row>
     <row r="10" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A10" t="s">
-        <v>88</v>
+        <v>77</v>
       </c>
       <c r="D10" t="s">
-        <v>151</v>
+        <v>51</v>
       </c>
       <c r="F10" t="s">
-        <v>89</v>
+        <v>78</v>
       </c>
       <c r="G10" t="s">
-        <v>90</v>
+        <v>79</v>
       </c>
       <c r="J10" t="s">
-        <v>91</v>
+        <v>80</v>
       </c>
     </row>
     <row r="11" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A11" t="s">
-        <v>88</v>
+        <v>77</v>
       </c>
       <c r="D11" t="s">
-        <v>150</v>
+        <v>66</v>
       </c>
       <c r="F11" t="s">
-        <v>92</v>
+        <v>81</v>
       </c>
       <c r="G11" t="s">
-        <v>93</v>
+        <v>82</v>
       </c>
     </row>
     <row r="12" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A12" t="s">
-        <v>88</v>
+        <v>77</v>
       </c>
       <c r="D12" t="s">
-        <v>152</v>
+        <v>83</v>
       </c>
       <c r="F12" t="s">
-        <v>94</v>
+        <v>84</v>
       </c>
       <c r="G12" t="s">
-        <v>95</v>
+        <v>85</v>
       </c>
     </row>
     <row r="13" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A13" t="s">
-        <v>96</v>
+        <v>86</v>
       </c>
       <c r="D13" t="s">
-        <v>151</v>
+        <v>51</v>
       </c>
       <c r="F13" t="s">
-        <v>97</v>
+        <v>87</v>
       </c>
       <c r="G13" t="s">
-        <v>98</v>
+        <v>88</v>
       </c>
     </row>
     <row r="14" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A14" t="s">
-        <v>96</v>
+        <v>86</v>
       </c>
       <c r="D14" t="s">
-        <v>152</v>
+        <v>83</v>
       </c>
       <c r="F14" t="s">
-        <v>99</v>
+        <v>89</v>
       </c>
       <c r="G14" t="s">
-        <v>100</v>
+        <v>90</v>
       </c>
     </row>
     <row r="15" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A15" t="s">
-        <v>96</v>
+        <v>86</v>
       </c>
       <c r="B15" s="4" t="s">
-        <v>154</v>
+        <v>91</v>
       </c>
       <c r="D15" t="s">
-        <v>155</v>
+        <v>92</v>
       </c>
       <c r="F15" t="s">
-        <v>101</v>
+        <v>93</v>
       </c>
       <c r="G15" t="s">
-        <v>102</v>
+        <v>94</v>
       </c>
     </row>
     <row r="16" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A16" t="s">
+        <v>86</v>
+      </c>
+      <c r="B16" t="s">
+        <v>95</v>
+      </c>
+      <c r="D16" t="s">
+        <v>92</v>
+      </c>
+      <c r="F16" t="s">
         <v>96</v>
       </c>
-      <c r="B16" t="s">
-        <v>153</v>
-      </c>
-      <c r="D16" t="s">
-        <v>155</v>
-      </c>
-      <c r="F16" t="s">
-        <v>103</v>
-      </c>
       <c r="G16" t="s">
-        <v>104</v>
+        <v>97</v>
       </c>
     </row>
     <row r="17" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A17" t="s">
-        <v>11</v>
+        <v>49</v>
       </c>
       <c r="D17" t="s">
-        <v>152</v>
+        <v>83</v>
       </c>
       <c r="F17" t="s">
-        <v>105</v>
+        <v>98</v>
       </c>
       <c r="G17" t="s">
-        <v>106</v>
+        <v>99</v>
       </c>
     </row>
     <row r="18" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A18" t="s">
-        <v>66</v>
+        <v>100</v>
       </c>
       <c r="D18" t="s">
-        <v>107</v>
+        <v>101</v>
       </c>
       <c r="F18" t="s">
-        <v>108</v>
+        <v>102</v>
       </c>
       <c r="G18" t="s">
-        <v>109</v>
+        <v>103</v>
       </c>
     </row>
     <row r="19" spans="1:9" x14ac:dyDescent="0.45">
       <c r="D19" t="s">
-        <v>110</v>
+        <v>104</v>
       </c>
       <c r="F19" t="s">
-        <v>111</v>
+        <v>105</v>
       </c>
       <c r="G19" t="s">
-        <v>112</v>
+        <v>106</v>
       </c>
     </row>
     <row r="20" spans="1:9" x14ac:dyDescent="0.45">
       <c r="D20" t="s">
-        <v>64</v>
+        <v>107</v>
       </c>
       <c r="F20" t="s">
-        <v>113</v>
+        <v>108</v>
       </c>
       <c r="G20" t="s">
-        <v>114</v>
+        <v>109</v>
       </c>
     </row>
     <row r="21" spans="1:9" x14ac:dyDescent="0.45">
       <c r="D21" t="s">
-        <v>115</v>
+        <v>110</v>
       </c>
       <c r="F21" t="s">
-        <v>116</v>
+        <v>111</v>
       </c>
       <c r="G21" t="s">
-        <v>117</v>
+        <v>112</v>
       </c>
     </row>
     <row r="22" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A22" t="s">
-        <v>11</v>
+        <v>49</v>
       </c>
       <c r="B22" s="4" t="s">
-        <v>148</v>
+        <v>113</v>
       </c>
       <c r="D22" t="s">
+        <v>114</v>
+      </c>
+      <c r="F22" t="s">
+        <v>115</v>
+      </c>
+      <c r="G22" t="s">
+        <v>116</v>
+      </c>
+      <c r="H22" t="s">
+        <v>117</v>
+      </c>
+      <c r="I22" t="s">
         <v>118</v>
-      </c>
-      <c r="F22" t="s">
-        <v>119</v>
-      </c>
-      <c r="G22" t="s">
-        <v>54</v>
-      </c>
-      <c r="H22" t="s">
-        <v>26</v>
-      </c>
-      <c r="I22" t="s">
-        <v>27</v>
       </c>
     </row>
     <row r="23" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A23" t="s">
-        <v>11</v>
+        <v>49</v>
       </c>
       <c r="B23" t="s">
+        <v>119</v>
+      </c>
+      <c r="D23" t="s">
+        <v>114</v>
+      </c>
+      <c r="F23" t="s">
         <v>120</v>
       </c>
-      <c r="D23" t="s">
-        <v>118</v>
-      </c>
-      <c r="F23" t="s">
+      <c r="G23" t="s">
         <v>121</v>
-      </c>
-      <c r="G23" t="s">
-        <v>122</v>
       </c>
     </row>
     <row r="24" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A24" t="s">
-        <v>11</v>
+        <v>49</v>
       </c>
       <c r="B24" t="s">
-        <v>53</v>
+        <v>122</v>
       </c>
       <c r="D24" t="s">
         <v>123</v>
       </c>
       <c r="F24" t="s">
-        <v>141</v>
+        <v>124</v>
       </c>
       <c r="G24" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="H24" t="s">
-        <v>26</v>
+        <v>117</v>
       </c>
       <c r="I24" t="s">
-        <v>27</v>
+        <v>118</v>
       </c>
     </row>
     <row r="25" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A25" t="s">
-        <v>11</v>
+        <v>49</v>
       </c>
       <c r="B25" t="s">
-        <v>52</v>
+        <v>126</v>
       </c>
       <c r="D25" t="s">
         <v>123</v>
       </c>
       <c r="F25" t="s">
-        <v>125</v>
+        <v>127</v>
       </c>
       <c r="G25" t="s">
-        <v>51</v>
+        <v>128</v>
       </c>
     </row>
     <row r="26" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A26" t="s">
-        <v>20</v>
+        <v>129</v>
       </c>
       <c r="B26" t="s">
-        <v>126</v>
+        <v>130</v>
       </c>
       <c r="F26" t="s">
-        <v>127</v>
+        <v>131</v>
       </c>
       <c r="G26" t="s">
-        <v>128</v>
+        <v>132</v>
       </c>
     </row>
     <row r="27" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A27" t="s">
-        <v>20</v>
+        <v>129</v>
       </c>
       <c r="B27" t="s">
-        <v>71</v>
+        <v>133</v>
       </c>
       <c r="F27" t="s">
-        <v>129</v>
+        <v>134</v>
       </c>
       <c r="G27" t="s">
-        <v>130</v>
+        <v>135</v>
       </c>
       <c r="H27" t="s">
-        <v>26</v>
+        <v>117</v>
       </c>
       <c r="I27" t="s">
-        <v>27</v>
+        <v>118</v>
       </c>
     </row>
     <row r="28" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A28" t="s">
-        <v>20</v>
+        <v>129</v>
       </c>
       <c r="B28" t="s">
-        <v>22</v>
+        <v>136</v>
       </c>
       <c r="F28" t="s">
-        <v>131</v>
+        <v>137</v>
       </c>
       <c r="G28" t="s">
-        <v>132</v>
-      </c>
-    </row>
-    <row r="33" spans="1:10" ht="17.25" thickBot="1" x14ac:dyDescent="0.55000000000000004">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="33" spans="1:10" ht="17.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A33" s="1" t="s">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="34" spans="1:10" ht="15" thickTop="1" thickBot="1" x14ac:dyDescent="0.5">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="34" spans="1:10" ht="15" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.5">
       <c r="A34" s="2" t="s">
-        <v>1</v>
+        <v>42</v>
       </c>
       <c r="B34" s="2" t="s">
-        <v>2</v>
+        <v>43</v>
       </c>
       <c r="C34" s="2" t="s">
-        <v>3</v>
+        <v>44</v>
       </c>
       <c r="D34" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="E34" s="2" t="s">
+        <v>46</v>
+      </c>
+      <c r="F34" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="E34" s="2" t="s">
+      <c r="G34" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="F34" s="2" t="s">
-        <v>6</v>
-      </c>
-      <c r="G34" s="2" t="s">
-        <v>7</v>
-      </c>
       <c r="H34" s="2" t="s">
+        <v>47</v>
+      </c>
+      <c r="I34" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="J34" s="2" t="s">
         <v>8</v>
-      </c>
-      <c r="I34" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="J34" s="2" t="s">
-        <v>10</v>
       </c>
     </row>
     <row r="35" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A35" t="s">
-        <v>29</v>
+        <v>139</v>
       </c>
       <c r="B35" t="s">
-        <v>30</v>
+        <v>140</v>
       </c>
       <c r="F35" t="s">
-        <v>28</v>
+        <v>141</v>
       </c>
     </row>
     <row r="36" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A36" t="s">
-        <v>31</v>
+        <v>142</v>
       </c>
       <c r="F36" t="s">
-        <v>32</v>
+        <v>143</v>
       </c>
     </row>
     <row r="37" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A37" t="s">
-        <v>49</v>
+        <v>144</v>
       </c>
       <c r="B37" t="s">
-        <v>50</v>
+        <v>145</v>
       </c>
       <c r="F37" t="s">
-        <v>63</v>
+        <v>146</v>
       </c>
     </row>
     <row r="38" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A38" t="s">
-        <v>49</v>
+        <v>144</v>
       </c>
       <c r="B38" t="s">
-        <v>61</v>
+        <v>147</v>
       </c>
       <c r="F38" t="s">
-        <v>62</v>
+        <v>148</v>
       </c>
     </row>
     <row r="39" spans="1:10" x14ac:dyDescent="0.45">
       <c r="B39" t="s">
-        <v>65</v>
+        <v>149</v>
       </c>
       <c r="F39" t="s">
-        <v>58</v>
+        <v>150</v>
       </c>
     </row>
     <row r="40" spans="1:10" x14ac:dyDescent="0.45">
       <c r="B40" t="s">
-        <v>59</v>
+        <v>151</v>
       </c>
       <c r="F40" t="s">
-        <v>60</v>
+        <v>152</v>
       </c>
     </row>
     <row r="41" spans="1:10" x14ac:dyDescent="0.45">
       <c r="B41" t="s">
-        <v>67</v>
+        <v>153</v>
       </c>
       <c r="F41" s="3" t="str">
         <f>LEFT(B41,9)</f>
@@ -6060,25 +6054,25 @@
     </row>
     <row r="42" spans="1:10" x14ac:dyDescent="0.45">
       <c r="B42" t="s">
-        <v>68</v>
+        <v>154</v>
       </c>
       <c r="F42" s="3" t="str">
-        <f t="shared" ref="F42:F43" si="0">LEFT(B42,9)</f>
+        <f>LEFT(B42,9)</f>
         <v>distr_won</v>
       </c>
     </row>
     <row r="43" spans="1:10" x14ac:dyDescent="0.45">
       <c r="B43" t="s">
-        <v>69</v>
+        <v>155</v>
       </c>
       <c r="F43" s="3" t="str">
-        <f t="shared" si="0"/>
+        <f>LEFT(B43,9)</f>
         <v>distr_wof</v>
       </c>
     </row>
     <row r="44" spans="1:10" x14ac:dyDescent="0.45">
       <c r="D44" t="s">
-        <v>23</v>
+        <v>156</v>
       </c>
       <c r="F44" s="3" t="str">
         <f>"hs_"&amp;D44</f>
@@ -6087,28 +6081,28 @@
     </row>
     <row r="45" spans="1:10" x14ac:dyDescent="0.45">
       <c r="D45" t="s">
-        <v>24</v>
+        <v>157</v>
       </c>
       <c r="F45" s="3" t="str">
-        <f t="shared" ref="F45:F47" si="1">"hs_"&amp;D45</f>
+        <f>"hs_"&amp;D45</f>
         <v>hs_hydro</v>
       </c>
     </row>
     <row r="46" spans="1:10" x14ac:dyDescent="0.45">
       <c r="D46" t="s">
-        <v>25</v>
+        <v>19</v>
       </c>
       <c r="F46" s="3" t="str">
-        <f t="shared" si="1"/>
+        <f>"hs_"&amp;D46</f>
         <v>hs_nuclear</v>
       </c>
     </row>
     <row r="47" spans="1:10" x14ac:dyDescent="0.45">
       <c r="D47" t="s">
-        <v>70</v>
+        <v>158</v>
       </c>
       <c r="F47" s="3" t="str">
-        <f t="shared" si="1"/>
+        <f>"hs_"&amp;D47</f>
         <v>hs_coal</v>
       </c>
     </row>

</xml_diff>